<commit_message>
commit before push due to moving seat
</commit_message>
<xml_diff>
--- a/figures/TCAD data.xlsx
+++ b/figures/TCAD data.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Desktop_offline\TCADtarget-manuscript-Jan\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A12C88AD-D5AD-4388-8C80-823B1B91A047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62B0EC5C-0760-4328-84B9-8F88BFADD4B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{6E1D205E-5548-4B10-8EA6-16E0E10C324F}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="1 V pgm 300-125-cryogenic raw" sheetId="4" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="24">
   <si>
     <t>time</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -106,11 +107,42 @@
     <t>model</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>300K</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ppp pattern</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>raw</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DVt from 0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DVt from 1V</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>125K</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>cry</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="178" formatCode="0.00000000E+00"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -150,7 +182,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -158,6 +190,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2011,6 +2046,1776 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62E00827-CB8A-4620-9DD2-40F83C23DE95}">
+  <dimension ref="A1:BI48"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.75" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" t="s">
+        <v>22</v>
+      </c>
+      <c r="L1" t="s">
+        <v>23</v>
+      </c>
+      <c r="R1">
+        <f>-1.21053305061</f>
+        <v>-1.21053305061</v>
+      </c>
+      <c r="S1">
+        <v>-1.21053305061</v>
+      </c>
+      <c r="T1">
+        <v>-1.210533085</v>
+      </c>
+      <c r="U1">
+        <v>-1.21053308501</v>
+      </c>
+      <c r="V1">
+        <v>-1.2105333435600001</v>
+      </c>
+      <c r="W1">
+        <v>-1.21053308501</v>
+      </c>
+      <c r="X1">
+        <v>-1.2105333437500001</v>
+      </c>
+      <c r="Y1">
+        <v>-1.21053308503</v>
+      </c>
+      <c r="Z1">
+        <v>-1.21053308526</v>
+      </c>
+      <c r="AA1">
+        <v>-1.21053353043</v>
+      </c>
+      <c r="AB1">
+        <v>-1.2105331105299999</v>
+      </c>
+      <c r="AC1">
+        <v>-1.2105335989499999</v>
+      </c>
+      <c r="AD1">
+        <v>-1.2105338542899999</v>
+      </c>
+      <c r="AE1">
+        <v>-1.2105343610999999</v>
+      </c>
+      <c r="AF1">
+        <v>-1.2105358204500001</v>
+      </c>
+      <c r="AG1">
+        <v>-1.21053892736</v>
+      </c>
+      <c r="AH1">
+        <v>-1.2105432680599999</v>
+      </c>
+      <c r="AI1">
+        <v>-1.2105533931100001</v>
+      </c>
+      <c r="AJ1">
+        <v>-1.2105736754300001</v>
+      </c>
+      <c r="AK1">
+        <v>-1.21061298957</v>
+      </c>
+      <c r="AL1">
+        <v>-1.2106896518700001</v>
+      </c>
+      <c r="AM1">
+        <v>-1.21083486941</v>
+      </c>
+      <c r="AN1">
+        <v>-1.21110029735</v>
+      </c>
+      <c r="AO1">
+        <v>-1.21156364201</v>
+      </c>
+      <c r="AP1">
+        <v>-1.2123318894699999</v>
+      </c>
+      <c r="AQ1">
+        <v>-1.21353997752</v>
+      </c>
+      <c r="AR1">
+        <v>-1.2153428958600001</v>
+      </c>
+      <c r="AS1">
+        <v>-1.2179015915</v>
+      </c>
+      <c r="AT1">
+        <v>-1.2213592658500001</v>
+      </c>
+      <c r="AU1">
+        <v>-1.22580667961</v>
+      </c>
+      <c r="AV1">
+        <v>-1.2342719196700001</v>
+      </c>
+      <c r="AW1">
+        <v>-1.2477149647500001</v>
+      </c>
+      <c r="AX1">
+        <v>-1.26248241977</v>
+      </c>
+      <c r="AY1">
+        <v>-1.27790400394</v>
+      </c>
+      <c r="AZ1">
+        <v>-1.3078410710299999</v>
+      </c>
+      <c r="BA1">
+        <v>-1.3290149843400001</v>
+      </c>
+      <c r="BB1">
+        <v>-1.3539236266900001</v>
+      </c>
+      <c r="BC1">
+        <v>-1.3750239037</v>
+      </c>
+      <c r="BD1">
+        <v>-1.3933387876000001</v>
+      </c>
+      <c r="BE1">
+        <v>-1.41557639992</v>
+      </c>
+      <c r="BF1">
+        <v>-1.44604972309</v>
+      </c>
+      <c r="BG1">
+        <v>-1.46504314619</v>
+      </c>
+      <c r="BH1">
+        <v>-1.48067604447</v>
+      </c>
+      <c r="BI1">
+        <v>-1.5019731222799999</v>
+      </c>
+    </row>
+    <row r="2" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" t="s">
+        <v>0</v>
+      </c>
+      <c r="L2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M2" t="s">
+        <v>20</v>
+      </c>
+      <c r="N2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>9.9999999999999998E-13</v>
+      </c>
+      <c r="B3">
+        <f>-1.21085737954</f>
+        <v>-1.2108573795399999</v>
+      </c>
+      <c r="C3">
+        <f t="shared" ref="C3:C47" si="0">B3-B$3</f>
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <f>1+C3</f>
+        <v>1</v>
+      </c>
+      <c r="F3" s="3">
+        <v>9.9999999999999998E-13</v>
+      </c>
+      <c r="G3">
+        <f>-1.21053305061</f>
+        <v>-1.21053305061</v>
+      </c>
+      <c r="H3">
+        <f t="shared" ref="H3:H47" si="1">G3-G$3</f>
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <f>1+H3</f>
+        <v>1</v>
+      </c>
+      <c r="K3" s="3">
+        <v>9.9999999999999998E-13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>0</v>
+      </c>
+      <c r="B4">
+        <v>-1.2108575775299999</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>-1.9798999995046529E-7</v>
+      </c>
+      <c r="D4">
+        <f>1+C4</f>
+        <v>0.99999980201000005</v>
+      </c>
+      <c r="F4" s="3">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>-1.21053305061</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <f>1+H4</f>
+        <v>1</v>
+      </c>
+      <c r="K4" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>9.9999999999999994E-12</v>
+      </c>
+      <c r="B5">
+        <v>-1.2108573793999999</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>1.4000001158365194E-10</v>
+      </c>
+      <c r="D5">
+        <f t="shared" ref="D5:D47" si="2">1+C5</f>
+        <v>1.00000000014</v>
+      </c>
+      <c r="F5" s="3">
+        <v>9.9999999999999994E-12</v>
+      </c>
+      <c r="G5">
+        <v>-1.210533085</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="1"/>
+        <v>-3.4389999958861495E-8</v>
+      </c>
+      <c r="I5">
+        <f t="shared" ref="I5:I47" si="3">1+H5</f>
+        <v>0.99999996561000004</v>
+      </c>
+      <c r="K5" s="3">
+        <v>9.9999999999999994E-12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>1E-10</v>
+      </c>
+      <c r="B6">
+        <v>-1.21085737531</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>4.2299999059025595E-9</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="2"/>
+        <v>1.0000000042299999</v>
+      </c>
+      <c r="F6" s="3">
+        <v>1E-10</v>
+      </c>
+      <c r="G6">
+        <v>-1.21053308501</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="1"/>
+        <v>-3.4399999959688898E-8</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="3"/>
+        <v>0.99999996560000004</v>
+      </c>
+      <c r="K6" s="3">
+        <v>1E-10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>1E-8</v>
+      </c>
+      <c r="B7">
+        <v>-1.2108576127699999</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="0"/>
+        <v>-2.332299999796561E-7</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="2"/>
+        <v>0.99999976677000002</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1E-8</v>
+      </c>
+      <c r="G7">
+        <v>-1.2105333435600001</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="1"/>
+        <v>-2.9295000003592975E-7</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="3"/>
+        <v>0.99999970704999996</v>
+      </c>
+      <c r="K7" s="3">
+        <v>1E-8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>9.9999999999999995E-8</v>
+      </c>
+      <c r="B8">
+        <v>-1.2108586510199999</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>-1.2714799999535842E-6</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="2"/>
+        <v>0.99999872852000005</v>
+      </c>
+      <c r="F8" s="3">
+        <v>9.9999999999999995E-8</v>
+      </c>
+      <c r="G8">
+        <v>-1.21053308501</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="1"/>
+        <v>-3.4399999959688898E-8</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="3"/>
+        <v>0.99999996560000004</v>
+      </c>
+      <c r="K8" s="3">
+        <v>9.9999999999999995E-8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="B9">
+        <v>-1.2108686231500001</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>-1.1243610000155613E-5</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="2"/>
+        <v>0.99998875638999984</v>
+      </c>
+      <c r="F9" s="3">
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="G9">
+        <v>-1.2105333437500001</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="1"/>
+        <v>-2.9314000005165042E-7</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="3"/>
+        <v>0.99999970685999995</v>
+      </c>
+      <c r="K9" s="3">
+        <v>9.9999999999999995E-7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="B10">
+        <v>-1.2109383394</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>-8.0959860000007211E-5</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="2"/>
+        <v>0.99991904013999999</v>
+      </c>
+      <c r="F10" s="3">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="G10">
+        <v>-1.21053308503</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="1"/>
+        <v>-3.4419999961343706E-8</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="3"/>
+        <v>0.99999996558000004</v>
+      </c>
+      <c r="K10" s="3">
+        <v>1.0000000000000001E-5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>1E-4</v>
+      </c>
+      <c r="B11">
+        <v>-1.21111774298</v>
+      </c>
+      <c r="C11">
+        <f t="shared" si="0"/>
+        <v>-2.6036344000002209E-4</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="2"/>
+        <v>0.99973963655999998</v>
+      </c>
+      <c r="F11" s="3">
+        <v>1E-4</v>
+      </c>
+      <c r="G11">
+        <v>-1.21053308526</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="1"/>
+        <v>-3.4649999980373991E-8</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="3"/>
+        <v>0.99999996535000002</v>
+      </c>
+      <c r="K11" s="3">
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
+        <v>1E-3</v>
+      </c>
+      <c r="B12">
+        <v>-1.2115532035900001</v>
+      </c>
+      <c r="C12">
+        <f t="shared" si="0"/>
+        <v>-6.958240500001267E-4</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="2"/>
+        <v>0.99930417594999987</v>
+      </c>
+      <c r="F12" s="3">
+        <v>1E-3</v>
+      </c>
+      <c r="G12">
+        <v>-1.21053353043</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="1"/>
+        <v>-4.7981999995450053E-7</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="3"/>
+        <v>0.99999952018000005</v>
+      </c>
+      <c r="K12" s="3">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B13">
+        <v>-1.2122793458200001</v>
+      </c>
+      <c r="C13">
+        <f t="shared" si="0"/>
+        <v>-1.4219662800001309E-3</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="2"/>
+        <v>0.99857803371999987</v>
+      </c>
+      <c r="F13" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="G13">
+        <v>-1.2105331105299999</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="1"/>
+        <v>-5.9919999850777117E-8</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="3"/>
+        <v>0.99999994008000015</v>
+      </c>
+      <c r="K13" s="3">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="14" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="B14">
+        <v>-1.21344702707</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="0"/>
+        <v>-2.5896475300000166E-3</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="2"/>
+        <v>0.99741035246999998</v>
+      </c>
+      <c r="F14" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="G14">
+        <v>-1.2105335989499999</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="1"/>
+        <v>-5.4833999985071102E-7</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="3"/>
+        <v>0.99999945166000015</v>
+      </c>
+      <c r="K14" s="3">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="B15">
+        <v>-1.2139142972200001</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="0"/>
+        <v>-3.0569176800001596E-3</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="2"/>
+        <v>0.99694308231999984</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="G15">
+        <v>-1.2105338542899999</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="1"/>
+        <v>-8.0367999988339989E-7</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="3"/>
+        <v>0.99999919632000012</v>
+      </c>
+      <c r="K15" s="3">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="B16">
+        <v>-1.2146313709600001</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="0"/>
+        <v>-3.7739914200001223E-3</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="2"/>
+        <v>0.99622600857999988</v>
+      </c>
+      <c r="F16" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="G16">
+        <v>-1.2105343610999999</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="1"/>
+        <v>-1.310489999850617E-6</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="3"/>
+        <v>0.99999868951000015</v>
+      </c>
+      <c r="K16" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
+        <v>1</v>
+      </c>
+      <c r="B17">
+        <v>-1.21522681108</v>
+      </c>
+      <c r="C17">
+        <f t="shared" si="0"/>
+        <v>-4.3694315400000239E-3</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="2"/>
+        <v>0.99563056845999998</v>
+      </c>
+      <c r="F17" s="3">
+        <v>1</v>
+      </c>
+      <c r="G17">
+        <v>-1.2105358204500001</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="1"/>
+        <v>-2.7698400000275569E-6</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="3"/>
+        <v>0.99999723015999997</v>
+      </c>
+      <c r="K17" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
+        <v>2</v>
+      </c>
+      <c r="B18">
+        <v>-1.21590102572</v>
+      </c>
+      <c r="C18">
+        <f t="shared" si="0"/>
+        <v>-5.0436461800000831E-3</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="2"/>
+        <v>0.99495635381999992</v>
+      </c>
+      <c r="F18" s="3">
+        <v>2</v>
+      </c>
+      <c r="G18">
+        <v>-1.21053892736</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="1"/>
+        <v>-5.8767499999667905E-6</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="3"/>
+        <v>0.99999412325000003</v>
+      </c>
+      <c r="K18" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="3">
+        <v>4</v>
+      </c>
+      <c r="B19">
+        <v>-1.21664939119</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="0"/>
+        <v>-5.7920116500000951E-3</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="2"/>
+        <v>0.9942079883499999</v>
+      </c>
+      <c r="F19" s="3">
+        <v>4</v>
+      </c>
+      <c r="G19">
+        <v>-1.2105432680599999</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="1"/>
+        <v>-1.0217449999849748E-5</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="3"/>
+        <v>0.99998978255000015</v>
+      </c>
+      <c r="K19" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" s="3">
+        <f>2*A19</f>
+        <v>8</v>
+      </c>
+      <c r="B20">
+        <v>-1.2174566757700001</v>
+      </c>
+      <c r="C20">
+        <f t="shared" si="0"/>
+        <v>-6.5992962300001068E-3</v>
+      </c>
+      <c r="D20">
+        <f t="shared" si="2"/>
+        <v>0.99340070376999989</v>
+      </c>
+      <c r="F20" s="3">
+        <f>2*F19</f>
+        <v>8</v>
+      </c>
+      <c r="G20">
+        <v>-1.2105533931100001</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="1"/>
+        <v>-2.0342500000047892E-5</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="3"/>
+        <v>0.99997965749999995</v>
+      </c>
+      <c r="K20" s="3">
+        <f>2*K19</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
+        <f t="shared" ref="A21:A47" si="4">2*A20</f>
+        <v>16</v>
+      </c>
+      <c r="B21">
+        <v>-1.21833466842</v>
+      </c>
+      <c r="C21">
+        <f t="shared" si="0"/>
+        <v>-7.4772888800000992E-3</v>
+      </c>
+      <c r="D21">
+        <f t="shared" si="2"/>
+        <v>0.9925227111199999</v>
+      </c>
+      <c r="F21" s="3">
+        <f t="shared" ref="F21:F47" si="5">2*F20</f>
+        <v>16</v>
+      </c>
+      <c r="G21">
+        <v>-1.2105736754300001</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="1"/>
+        <v>-4.0624820000001449E-5</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="3"/>
+        <v>0.99995937518</v>
+      </c>
+      <c r="K21" s="3">
+        <f t="shared" ref="K21:K47" si="6">2*K20</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22" s="3">
+        <f t="shared" si="4"/>
+        <v>32</v>
+      </c>
+      <c r="B22">
+        <v>-1.21929042945</v>
+      </c>
+      <c r="C22">
+        <f t="shared" si="0"/>
+        <v>-8.4330499100000456E-3</v>
+      </c>
+      <c r="D22">
+        <f t="shared" si="2"/>
+        <v>0.99156695008999995</v>
+      </c>
+      <c r="F22" s="3">
+        <f t="shared" si="5"/>
+        <v>32</v>
+      </c>
+      <c r="G22">
+        <v>-1.21061298957</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="1"/>
+        <v>-7.9938959999914516E-5</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="3"/>
+        <v>0.99992006104000009</v>
+      </c>
+      <c r="K22" s="3">
+        <f t="shared" si="6"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" s="3">
+        <f t="shared" si="4"/>
+        <v>64</v>
+      </c>
+      <c r="B23">
+        <v>-1.2203125752399999</v>
+      </c>
+      <c r="C23">
+        <f t="shared" si="0"/>
+        <v>-9.4551956999999742E-3</v>
+      </c>
+      <c r="D23">
+        <f t="shared" si="2"/>
+        <v>0.99054480430000003</v>
+      </c>
+      <c r="F23" s="3">
+        <f t="shared" si="5"/>
+        <v>64</v>
+      </c>
+      <c r="G23">
+        <v>-1.2106896518700001</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="1"/>
+        <v>-1.5660126000005548E-4</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="3"/>
+        <v>0.99984339873999994</v>
+      </c>
+      <c r="K23" s="3">
+        <f t="shared" si="6"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" s="3">
+        <f t="shared" si="4"/>
+        <v>128</v>
+      </c>
+      <c r="B24">
+        <v>-1.2214018093600001</v>
+      </c>
+      <c r="C24">
+        <f t="shared" si="0"/>
+        <v>-1.0544429820000145E-2</v>
+      </c>
+      <c r="D24">
+        <f t="shared" si="2"/>
+        <v>0.98945557017999985</v>
+      </c>
+      <c r="F24" s="3">
+        <f t="shared" si="5"/>
+        <v>128</v>
+      </c>
+      <c r="G24">
+        <v>-1.21083486941</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="1"/>
+        <v>-3.018187999999089E-4</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="3"/>
+        <v>0.99969818120000009</v>
+      </c>
+      <c r="K24" s="3">
+        <f t="shared" si="6"/>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" s="3">
+        <f t="shared" si="4"/>
+        <v>256</v>
+      </c>
+      <c r="B25">
+        <v>-1.22255927744</v>
+      </c>
+      <c r="C25">
+        <f t="shared" si="0"/>
+        <v>-1.1701897900000091E-2</v>
+      </c>
+      <c r="D25">
+        <f t="shared" si="2"/>
+        <v>0.98829810209999991</v>
+      </c>
+      <c r="F25" s="3">
+        <f t="shared" si="5"/>
+        <v>256</v>
+      </c>
+      <c r="G25">
+        <v>-1.21110029735</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="1"/>
+        <v>-5.6724673999997144E-4</v>
+      </c>
+      <c r="I25">
+        <f t="shared" si="3"/>
+        <v>0.99943275326000003</v>
+      </c>
+      <c r="K25" s="3">
+        <f t="shared" si="6"/>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26" s="3">
+        <f t="shared" si="4"/>
+        <v>512</v>
+      </c>
+      <c r="B26">
+        <v>-1.22377873478</v>
+      </c>
+      <c r="C26">
+        <f t="shared" si="0"/>
+        <v>-1.2921355240000043E-2</v>
+      </c>
+      <c r="D26">
+        <f t="shared" si="2"/>
+        <v>0.98707864475999996</v>
+      </c>
+      <c r="F26" s="3">
+        <f t="shared" si="5"/>
+        <v>512</v>
+      </c>
+      <c r="G26">
+        <v>-1.21156364201</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="1"/>
+        <v>-1.0305913999999472E-3</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="3"/>
+        <v>0.99896940860000005</v>
+      </c>
+      <c r="K26" s="3">
+        <f t="shared" si="6"/>
+        <v>512</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27" s="3">
+        <f t="shared" si="4"/>
+        <v>1024</v>
+      </c>
+      <c r="B27">
+        <v>-1.2250586692800001</v>
+      </c>
+      <c r="C27">
+        <f t="shared" si="0"/>
+        <v>-1.4201289740000123E-2</v>
+      </c>
+      <c r="D27">
+        <f t="shared" si="2"/>
+        <v>0.98579871025999988</v>
+      </c>
+      <c r="F27" s="3">
+        <f t="shared" si="5"/>
+        <v>1024</v>
+      </c>
+      <c r="G27">
+        <v>-1.2123318894699999</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="1"/>
+        <v>-1.7988388599998739E-3</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="3"/>
+        <v>0.99820116114000013</v>
+      </c>
+      <c r="K27" s="3">
+        <f t="shared" si="6"/>
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28" s="3">
+        <f t="shared" si="4"/>
+        <v>2048</v>
+      </c>
+      <c r="B28">
+        <v>-1.22639668161</v>
+      </c>
+      <c r="C28">
+        <f t="shared" si="0"/>
+        <v>-1.5539302070000094E-2</v>
+      </c>
+      <c r="D28">
+        <f t="shared" si="2"/>
+        <v>0.98446069792999991</v>
+      </c>
+      <c r="F28" s="3">
+        <f t="shared" si="5"/>
+        <v>2048</v>
+      </c>
+      <c r="G28">
+        <v>-1.21353997752</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="1"/>
+        <v>-3.0069269099999296E-3</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="3"/>
+        <v>0.99699307309000007</v>
+      </c>
+      <c r="K28" s="3">
+        <f t="shared" si="6"/>
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29" s="3">
+        <f t="shared" si="4"/>
+        <v>4096</v>
+      </c>
+      <c r="B29">
+        <v>-1.22779076002</v>
+      </c>
+      <c r="C29">
+        <f t="shared" si="0"/>
+        <v>-1.6933380480000038E-2</v>
+      </c>
+      <c r="D29">
+        <f t="shared" si="2"/>
+        <v>0.98306661951999996</v>
+      </c>
+      <c r="F29" s="3">
+        <f t="shared" si="5"/>
+        <v>4096</v>
+      </c>
+      <c r="G29">
+        <v>-1.2153428958600001</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="1"/>
+        <v>-4.8098452500000555E-3</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="3"/>
+        <v>0.99519015474999994</v>
+      </c>
+      <c r="K29" s="3">
+        <f t="shared" si="6"/>
+        <v>4096</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" s="3">
+        <f t="shared" si="4"/>
+        <v>8192</v>
+      </c>
+      <c r="B30">
+        <v>-1.22999274846</v>
+      </c>
+      <c r="C30">
+        <f t="shared" si="0"/>
+        <v>-1.9135368920000007E-2</v>
+      </c>
+      <c r="D30">
+        <f t="shared" si="2"/>
+        <v>0.98086463107999999</v>
+      </c>
+      <c r="F30" s="3">
+        <f t="shared" si="5"/>
+        <v>8192</v>
+      </c>
+      <c r="G30">
+        <v>-1.2179015915</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="1"/>
+        <v>-7.3685408899999416E-3</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="3"/>
+        <v>0.99263145911000006</v>
+      </c>
+      <c r="K30" s="3">
+        <f t="shared" si="6"/>
+        <v>8192</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" s="3">
+        <f t="shared" si="4"/>
+        <v>16384</v>
+      </c>
+      <c r="B31">
+        <v>-1.2332103886000001</v>
+      </c>
+      <c r="C31">
+        <f t="shared" si="0"/>
+        <v>-2.2353009060000151E-2</v>
+      </c>
+      <c r="D31">
+        <f t="shared" si="2"/>
+        <v>0.97764699093999985</v>
+      </c>
+      <c r="F31" s="3">
+        <f t="shared" si="5"/>
+        <v>16384</v>
+      </c>
+      <c r="G31">
+        <v>-1.2213592658500001</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="1"/>
+        <v>-1.0826215240000048E-2</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="3"/>
+        <v>0.98917378475999995</v>
+      </c>
+      <c r="K31" s="3">
+        <f t="shared" si="6"/>
+        <v>16384</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
+        <f t="shared" si="4"/>
+        <v>32768</v>
+      </c>
+      <c r="B32">
+        <v>-1.23654973139</v>
+      </c>
+      <c r="C32">
+        <f t="shared" si="0"/>
+        <v>-2.5692351850000072E-2</v>
+      </c>
+      <c r="D32">
+        <f t="shared" si="2"/>
+        <v>0.97430764814999993</v>
+      </c>
+      <c r="F32" s="3">
+        <f t="shared" si="5"/>
+        <v>32768</v>
+      </c>
+      <c r="G32">
+        <v>-1.22580667961</v>
+      </c>
+      <c r="H32">
+        <f t="shared" si="1"/>
+        <v>-1.5273628999999955E-2</v>
+      </c>
+      <c r="I32">
+        <f t="shared" si="3"/>
+        <v>0.98472637100000004</v>
+      </c>
+      <c r="K32" s="3">
+        <f t="shared" si="6"/>
+        <v>32768</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="3">
+        <f t="shared" si="4"/>
+        <v>65536</v>
+      </c>
+      <c r="B33">
+        <v>-1.2400242341600001</v>
+      </c>
+      <c r="C33">
+        <f t="shared" si="0"/>
+        <v>-2.9166854620000127E-2</v>
+      </c>
+      <c r="D33">
+        <f t="shared" si="2"/>
+        <v>0.97083314537999987</v>
+      </c>
+      <c r="F33" s="3">
+        <f t="shared" si="5"/>
+        <v>65536</v>
+      </c>
+      <c r="G33">
+        <v>-1.2342719196700001</v>
+      </c>
+      <c r="H33">
+        <f t="shared" si="1"/>
+        <v>-2.3738869060000001E-2</v>
+      </c>
+      <c r="I33">
+        <f t="shared" si="3"/>
+        <v>0.97626113094</v>
+      </c>
+      <c r="K33" s="3">
+        <f t="shared" si="6"/>
+        <v>65536</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" s="3">
+        <f t="shared" si="4"/>
+        <v>131072</v>
+      </c>
+      <c r="B34">
+        <v>-1.24366373293</v>
+      </c>
+      <c r="C34">
+        <f t="shared" si="0"/>
+        <v>-3.2806353390000043E-2</v>
+      </c>
+      <c r="D34">
+        <f t="shared" si="2"/>
+        <v>0.96719364660999996</v>
+      </c>
+      <c r="F34" s="3">
+        <f t="shared" si="5"/>
+        <v>131072</v>
+      </c>
+      <c r="G34">
+        <v>-1.2477149647500001</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="1"/>
+        <v>-3.718191414000005E-2</v>
+      </c>
+      <c r="I34">
+        <f t="shared" si="3"/>
+        <v>0.96281808585999995</v>
+      </c>
+      <c r="K34" s="3">
+        <f t="shared" si="6"/>
+        <v>131072</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" s="3">
+        <f t="shared" si="4"/>
+        <v>262144</v>
+      </c>
+      <c r="B35">
+        <v>-1.2475180344200001</v>
+      </c>
+      <c r="C35">
+        <f t="shared" si="0"/>
+        <v>-3.6660654880000143E-2</v>
+      </c>
+      <c r="D35">
+        <f t="shared" si="2"/>
+        <v>0.96333934511999986</v>
+      </c>
+      <c r="F35" s="3">
+        <f t="shared" si="5"/>
+        <v>262144</v>
+      </c>
+      <c r="G35">
+        <v>-1.26248241977</v>
+      </c>
+      <c r="H35">
+        <f t="shared" si="1"/>
+        <v>-5.1949369159999925E-2</v>
+      </c>
+      <c r="I35">
+        <f t="shared" si="3"/>
+        <v>0.94805063084000007</v>
+      </c>
+      <c r="K35" s="3">
+        <f t="shared" si="6"/>
+        <v>262144</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" s="3">
+        <f t="shared" si="4"/>
+        <v>524288</v>
+      </c>
+      <c r="B36">
+        <v>-1.2516457401800001</v>
+      </c>
+      <c r="C36">
+        <f t="shared" si="0"/>
+        <v>-4.0788360640000132E-2</v>
+      </c>
+      <c r="D36">
+        <f t="shared" si="2"/>
+        <v>0.95921163935999987</v>
+      </c>
+      <c r="F36" s="3">
+        <f t="shared" si="5"/>
+        <v>524288</v>
+      </c>
+      <c r="G36">
+        <v>-1.27790400394</v>
+      </c>
+      <c r="H36">
+        <f t="shared" si="1"/>
+        <v>-6.7370953329999983E-2</v>
+      </c>
+      <c r="I36">
+        <f t="shared" si="3"/>
+        <v>0.93262904667000002</v>
+      </c>
+      <c r="K36" s="3">
+        <f t="shared" si="6"/>
+        <v>524288</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" s="3">
+        <f t="shared" si="4"/>
+        <v>1048576</v>
+      </c>
+      <c r="B37">
+        <v>-1.2561012808700001</v>
+      </c>
+      <c r="C37">
+        <f t="shared" si="0"/>
+        <v>-4.5243901330000114E-2</v>
+      </c>
+      <c r="D37">
+        <f t="shared" si="2"/>
+        <v>0.95475609866999989</v>
+      </c>
+      <c r="F37" s="3">
+        <f t="shared" si="5"/>
+        <v>1048576</v>
+      </c>
+      <c r="K37" s="3">
+        <f t="shared" si="6"/>
+        <v>1048576</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" s="3">
+        <f t="shared" si="4"/>
+        <v>2097152</v>
+      </c>
+      <c r="B38">
+        <v>-1.2609020798399999</v>
+      </c>
+      <c r="C38">
+        <f t="shared" si="0"/>
+        <v>-5.0044700299999967E-2</v>
+      </c>
+      <c r="D38">
+        <f t="shared" si="2"/>
+        <v>0.94995529970000003</v>
+      </c>
+      <c r="F38" s="3">
+        <f t="shared" si="5"/>
+        <v>2097152</v>
+      </c>
+      <c r="G38">
+        <v>-1.3078410710299999</v>
+      </c>
+      <c r="H38">
+        <f t="shared" si="1"/>
+        <v>-9.7308020419999863E-2</v>
+      </c>
+      <c r="I38">
+        <f t="shared" si="3"/>
+        <v>0.90269197958000014</v>
+      </c>
+      <c r="K38" s="3">
+        <f t="shared" si="6"/>
+        <v>2097152</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" s="3">
+        <f t="shared" si="4"/>
+        <v>4194304</v>
+      </c>
+      <c r="B39">
+        <v>-1.2659934478099999</v>
+      </c>
+      <c r="C39">
+        <f t="shared" si="0"/>
+        <v>-5.5136068269999949E-2</v>
+      </c>
+      <c r="D39">
+        <f t="shared" si="2"/>
+        <v>0.94486393173000005</v>
+      </c>
+      <c r="F39" s="3">
+        <f t="shared" si="5"/>
+        <v>4194304</v>
+      </c>
+      <c r="G39">
+        <v>-1.3290149843400001</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="1"/>
+        <v>-0.11848193373000004</v>
+      </c>
+      <c r="I39">
+        <f t="shared" si="3"/>
+        <v>0.88151806626999996</v>
+      </c>
+      <c r="K39" s="3">
+        <f t="shared" si="6"/>
+        <v>4194304</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" s="3">
+        <f t="shared" si="4"/>
+        <v>8388608</v>
+      </c>
+      <c r="B40">
+        <v>-1.27123021886</v>
+      </c>
+      <c r="C40">
+        <f t="shared" si="0"/>
+        <v>-6.0372839320000038E-2</v>
+      </c>
+      <c r="D40">
+        <f t="shared" si="2"/>
+        <v>0.93962716067999996</v>
+      </c>
+      <c r="F40" s="3">
+        <f t="shared" si="5"/>
+        <v>8388608</v>
+      </c>
+      <c r="G40">
+        <v>-1.3539236266900001</v>
+      </c>
+      <c r="H40">
+        <f t="shared" si="1"/>
+        <v>-0.14339057608000005</v>
+      </c>
+      <c r="I40">
+        <f t="shared" si="3"/>
+        <v>0.85660942391999995</v>
+      </c>
+      <c r="K40" s="3">
+        <f t="shared" si="6"/>
+        <v>8388608</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" s="3">
+        <f t="shared" si="4"/>
+        <v>16777216</v>
+      </c>
+      <c r="B41">
+        <v>-1.27640506393</v>
+      </c>
+      <c r="C41">
+        <f t="shared" si="0"/>
+        <v>-6.5547684390000027E-2</v>
+      </c>
+      <c r="D41">
+        <f t="shared" si="2"/>
+        <v>0.93445231560999997</v>
+      </c>
+      <c r="F41" s="3">
+        <f t="shared" si="5"/>
+        <v>16777216</v>
+      </c>
+      <c r="G41">
+        <v>-1.3750239037</v>
+      </c>
+      <c r="H41">
+        <f t="shared" si="1"/>
+        <v>-0.16449085309</v>
+      </c>
+      <c r="I41">
+        <f t="shared" si="3"/>
+        <v>0.83550914691</v>
+      </c>
+      <c r="K41" s="3">
+        <f t="shared" si="6"/>
+        <v>16777216</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" s="3">
+        <f t="shared" si="4"/>
+        <v>33554432</v>
+      </c>
+      <c r="B42">
+        <v>-1.28131098782</v>
+      </c>
+      <c r="C42">
+        <f t="shared" si="0"/>
+        <v>-7.0453608280000024E-2</v>
+      </c>
+      <c r="D42">
+        <f t="shared" si="2"/>
+        <v>0.92954639171999998</v>
+      </c>
+      <c r="F42" s="3">
+        <f t="shared" si="5"/>
+        <v>33554432</v>
+      </c>
+      <c r="G42">
+        <v>-1.3933387876000001</v>
+      </c>
+      <c r="H42">
+        <f t="shared" si="1"/>
+        <v>-0.18280573699000002</v>
+      </c>
+      <c r="I42">
+        <f t="shared" si="3"/>
+        <v>0.81719426300999998</v>
+      </c>
+      <c r="K42" s="3">
+        <f t="shared" si="6"/>
+        <v>33554432</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" s="3">
+        <f t="shared" si="4"/>
+        <v>67108864</v>
+      </c>
+      <c r="B43">
+        <v>-1.2858112295499999</v>
+      </c>
+      <c r="C43">
+        <f t="shared" si="0"/>
+        <v>-7.4953850009999989E-2</v>
+      </c>
+      <c r="D43">
+        <f t="shared" si="2"/>
+        <v>0.92504614999000001</v>
+      </c>
+      <c r="F43" s="3">
+        <f t="shared" si="5"/>
+        <v>67108864</v>
+      </c>
+      <c r="G43">
+        <v>-1.41557639992</v>
+      </c>
+      <c r="H43">
+        <f t="shared" si="1"/>
+        <v>-0.2050433493099999</v>
+      </c>
+      <c r="I43">
+        <f t="shared" si="3"/>
+        <v>0.7949566506900001</v>
+      </c>
+      <c r="K43" s="3">
+        <f t="shared" si="6"/>
+        <v>67108864</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" s="3">
+        <f t="shared" si="4"/>
+        <v>134217728</v>
+      </c>
+      <c r="B44">
+        <v>-1.2950270048900001</v>
+      </c>
+      <c r="C44">
+        <f t="shared" si="0"/>
+        <v>-8.4169625350000166E-2</v>
+      </c>
+      <c r="D44">
+        <f t="shared" si="2"/>
+        <v>0.91583037464999983</v>
+      </c>
+      <c r="F44" s="3">
+        <f t="shared" si="5"/>
+        <v>134217728</v>
+      </c>
+      <c r="G44">
+        <v>-1.44604972309</v>
+      </c>
+      <c r="H44">
+        <f t="shared" si="1"/>
+        <v>-0.23551667247999997</v>
+      </c>
+      <c r="I44">
+        <f t="shared" si="3"/>
+        <v>0.76448332752000003</v>
+      </c>
+      <c r="K44" s="3">
+        <f t="shared" si="6"/>
+        <v>134217728</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" s="3">
+        <f t="shared" si="4"/>
+        <v>268435456</v>
+      </c>
+      <c r="B45">
+        <v>-1.2985161512900001</v>
+      </c>
+      <c r="C45">
+        <f t="shared" si="0"/>
+        <v>-8.7658771750000142E-2</v>
+      </c>
+      <c r="D45">
+        <f t="shared" si="2"/>
+        <v>0.91234122824999986</v>
+      </c>
+      <c r="F45" s="3">
+        <f t="shared" si="5"/>
+        <v>268435456</v>
+      </c>
+      <c r="G45">
+        <v>-1.46504314619</v>
+      </c>
+      <c r="H45">
+        <f t="shared" si="1"/>
+        <v>-0.25451009557999993</v>
+      </c>
+      <c r="I45">
+        <f t="shared" si="3"/>
+        <v>0.74548990442000007</v>
+      </c>
+      <c r="K45" s="3">
+        <f t="shared" si="6"/>
+        <v>268435456</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" s="3">
+        <f t="shared" si="4"/>
+        <v>536870912</v>
+      </c>
+      <c r="B46">
+        <v>-1.30183358197</v>
+      </c>
+      <c r="C46">
+        <f t="shared" si="0"/>
+        <v>-9.0976202430000042E-2</v>
+      </c>
+      <c r="D46">
+        <f t="shared" si="2"/>
+        <v>0.90902379756999996</v>
+      </c>
+      <c r="F46" s="3">
+        <f t="shared" si="5"/>
+        <v>536870912</v>
+      </c>
+      <c r="G46">
+        <v>-1.48067604447</v>
+      </c>
+      <c r="H46">
+        <f t="shared" si="1"/>
+        <v>-0.27014299385999996</v>
+      </c>
+      <c r="I46">
+        <f t="shared" si="3"/>
+        <v>0.72985700614000004</v>
+      </c>
+      <c r="K46" s="3">
+        <f t="shared" si="6"/>
+        <v>536870912</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" s="3">
+        <f t="shared" si="4"/>
+        <v>1073741824</v>
+      </c>
+      <c r="B47">
+        <v>-1.30533086595</v>
+      </c>
+      <c r="C47">
+        <f t="shared" si="0"/>
+        <v>-9.4473486410000085E-2</v>
+      </c>
+      <c r="D47">
+        <f t="shared" si="2"/>
+        <v>0.90552651358999992</v>
+      </c>
+      <c r="F47" s="3">
+        <f t="shared" si="5"/>
+        <v>1073741824</v>
+      </c>
+      <c r="G47">
+        <v>-1.5019731222799999</v>
+      </c>
+      <c r="H47">
+        <f t="shared" si="1"/>
+        <v>-0.29144007166999986</v>
+      </c>
+      <c r="I47">
+        <f t="shared" si="3"/>
+        <v>0.70855992833000014</v>
+      </c>
+      <c r="K47" s="3">
+        <f t="shared" si="6"/>
+        <v>1073741824</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" s="1"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61E7C826-F786-4EE7-9C76-F06B5176B29E}">
   <dimension ref="A1:R47"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -4283,7 +6088,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C4C1E0D-2AEE-4A7F-82EA-F9A1189D6A82}">
   <dimension ref="A1:K1050"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -16549,7 +18354,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0971B89F-4BB2-40B3-A650-BC46BAF40E7C}">
   <dimension ref="A1:P162"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
figure 2 simulation ongoing: cryogenic - room temp figure calibration to Refaldi by 3/6/8 scale, 3/3.5/4/4.5/5 cryogenic modeling matching will be done soon.
</commit_message>
<xml_diff>
--- a/figures/TCAD data.xlsx
+++ b/figures/TCAD data.xlsx
@@ -5,18 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Desktop_offline\TCADtarget-manuscript-Jan\figures\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshs\Desktop\local-laptop\EDLtarget-manuscript-December\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62B0EC5C-0760-4328-84B9-8F88BFADD4B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEA71504-E459-4B0E-B22C-324A39F91EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{6E1D205E-5548-4B10-8EA6-16E0E10C324F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6E1D205E-5548-4B10-8EA6-16E0E10C324F}"/>
   </bookViews>
   <sheets>
     <sheet name="1 V pgm 300-125-cryogenic raw" sheetId="4" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId4"/>
+    <sheet name="cryogenic 3 3.5 4 5" sheetId="5" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId4"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="24">
   <si>
     <t>time</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -141,7 +142,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="178" formatCode="0.00000000E+00"/>
+    <numFmt numFmtId="176" formatCode="0.00000000E+00"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -192,7 +193,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -3816,6 +3817,1851 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB8F665F-4B87-445E-8D0D-37A1126372C0}">
+  <dimension ref="B2:I72"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B3" s="1">
+        <v>9.9999999999999998E-13</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D3" s="1">
+        <v>9.9999999999999998E-13</v>
+      </c>
+      <c r="E3" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F3" s="1">
+        <v>9.9999999999999998E-13</v>
+      </c>
+      <c r="G3" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H3" s="1">
+        <v>9.9999999999999998E-13</v>
+      </c>
+      <c r="I3" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B4" s="1">
+        <v>3.0000000000000001E-12</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D4" s="1">
+        <v>3.0000000000000001E-12</v>
+      </c>
+      <c r="E4" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F4" s="1">
+        <v>3.0000000000000001E-12</v>
+      </c>
+      <c r="G4" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H4" s="1">
+        <v>3.0000000000000001E-12</v>
+      </c>
+      <c r="I4" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B5" s="1">
+        <v>7.0000000000000001E-12</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D5" s="1">
+        <v>7.0000000000000001E-12</v>
+      </c>
+      <c r="E5" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F5" s="1">
+        <v>7.0000000000000001E-12</v>
+      </c>
+      <c r="G5" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H5" s="1">
+        <v>7.0000000000000001E-12</v>
+      </c>
+      <c r="I5" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B6" s="1">
+        <v>9.9999999999999994E-12</v>
+      </c>
+      <c r="C6" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D6" s="1">
+        <v>9.9999999999999994E-12</v>
+      </c>
+      <c r="E6" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F6" s="1">
+        <v>9.9999999999999994E-12</v>
+      </c>
+      <c r="G6" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H6" s="1">
+        <v>9.9999999999999994E-12</v>
+      </c>
+      <c r="I6" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B7" s="1">
+        <v>1.7999999999999999E-11</v>
+      </c>
+      <c r="C7" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D7" s="1">
+        <v>1.7999999999999999E-11</v>
+      </c>
+      <c r="E7" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F7" s="1">
+        <v>1.7999999999999999E-11</v>
+      </c>
+      <c r="G7" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H7" s="1">
+        <v>1.7999999999999999E-11</v>
+      </c>
+      <c r="I7" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B8" s="1">
+        <v>3.3999999999999999E-11</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D8" s="1">
+        <v>3.3999999999999999E-11</v>
+      </c>
+      <c r="E8" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F8" s="1">
+        <v>3.3999999999999999E-11</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H8" s="1">
+        <v>3.3999999999999999E-11</v>
+      </c>
+      <c r="I8" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B9" s="1">
+        <v>6.6000000000000005E-11</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D9" s="1">
+        <v>6.6000000000000005E-11</v>
+      </c>
+      <c r="E9" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F9" s="1">
+        <v>6.6000000000000005E-11</v>
+      </c>
+      <c r="G9" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H9" s="1">
+        <v>6.6000000000000005E-11</v>
+      </c>
+      <c r="I9" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B10" s="1">
+        <v>1E-10</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1E-10</v>
+      </c>
+      <c r="E10" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F10" s="1">
+        <v>1E-10</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H10" s="1">
+        <v>1E-10</v>
+      </c>
+      <c r="I10" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B11" s="1">
+        <v>2.0751743999999999E-10</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D11" s="1">
+        <v>2.0751743999999999E-10</v>
+      </c>
+      <c r="E11" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F11" s="1">
+        <v>2.0751743999999999E-10</v>
+      </c>
+      <c r="G11" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H11" s="1">
+        <v>2.0751743999999999E-10</v>
+      </c>
+      <c r="I11" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B12" s="1">
+        <v>4.2255232E-10</v>
+      </c>
+      <c r="C12" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D12" s="1">
+        <v>4.2255232E-10</v>
+      </c>
+      <c r="E12" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F12" s="1">
+        <v>4.2255232E-10</v>
+      </c>
+      <c r="G12" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H12" s="1">
+        <v>4.2255232E-10</v>
+      </c>
+      <c r="I12" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B13" s="1">
+        <v>8.5262207999999996E-10</v>
+      </c>
+      <c r="C13" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D13" s="1">
+        <v>8.5262207999999996E-10</v>
+      </c>
+      <c r="E13" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F13" s="1">
+        <v>8.5262207999999996E-10</v>
+      </c>
+      <c r="G13" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H13" s="1">
+        <v>8.5262207999999996E-10</v>
+      </c>
+      <c r="I13" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B14" s="1">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="C14" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D14" s="1">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="E14" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F14" s="1">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="G14" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H14" s="1">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="I14" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B15" s="1">
+        <v>1.8601395E-9</v>
+      </c>
+      <c r="C15" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D15" s="1">
+        <v>1.8601395E-9</v>
+      </c>
+      <c r="E15" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F15" s="1">
+        <v>1.8601395E-9</v>
+      </c>
+      <c r="G15" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H15" s="1">
+        <v>1.8601395E-9</v>
+      </c>
+      <c r="I15" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B16" s="1">
+        <v>3.5804185999999999E-9</v>
+      </c>
+      <c r="C16" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D16" s="1">
+        <v>3.5804185999999999E-9</v>
+      </c>
+      <c r="E16" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F16" s="1">
+        <v>3.5804185999999999E-9</v>
+      </c>
+      <c r="G16" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H16" s="1">
+        <v>3.5804185999999999E-9</v>
+      </c>
+      <c r="I16" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B17" s="1">
+        <v>7.0209766999999997E-9</v>
+      </c>
+      <c r="C17" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D17" s="1">
+        <v>7.0209766999999997E-9</v>
+      </c>
+      <c r="E17" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F17" s="1">
+        <v>7.0209766999999997E-9</v>
+      </c>
+      <c r="G17" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H17" s="1">
+        <v>7.0209766999999997E-9</v>
+      </c>
+      <c r="I17" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B18" s="1">
+        <v>1E-8</v>
+      </c>
+      <c r="C18" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1E-8</v>
+      </c>
+      <c r="E18" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F18" s="1">
+        <v>1E-8</v>
+      </c>
+      <c r="G18" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H18" s="1">
+        <v>1E-8</v>
+      </c>
+      <c r="I18" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B19" s="1">
+        <v>1.6881116000000001E-8</v>
+      </c>
+      <c r="C19" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D19" s="1">
+        <v>1.6881116000000001E-8</v>
+      </c>
+      <c r="E19" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F19" s="1">
+        <v>1.6881116000000001E-8</v>
+      </c>
+      <c r="G19" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H19" s="1">
+        <v>1.6881116000000001E-8</v>
+      </c>
+      <c r="I19" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B20" s="1">
+        <v>3.0643349000000001E-8</v>
+      </c>
+      <c r="C20" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D20" s="1">
+        <v>3.0643349000000001E-8</v>
+      </c>
+      <c r="E20" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F20" s="1">
+        <v>3.0643349000000001E-8</v>
+      </c>
+      <c r="G20" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H20" s="1">
+        <v>3.0643349000000001E-8</v>
+      </c>
+      <c r="I20" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B21" s="1">
+        <v>5.8167812999999998E-8</v>
+      </c>
+      <c r="C21" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D21" s="1">
+        <v>5.8167812999999998E-8</v>
+      </c>
+      <c r="E21" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F21" s="1">
+        <v>5.8167812999999998E-8</v>
+      </c>
+      <c r="G21" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H21" s="1">
+        <v>5.8167812999999998E-8</v>
+      </c>
+      <c r="I21" s="1">
+        <v>1.2137459E+19</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B22" s="1">
+        <v>9.9999999999999995E-8</v>
+      </c>
+      <c r="C22" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D22" s="1">
+        <v>9.9999999999999995E-8</v>
+      </c>
+      <c r="E22" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F22" s="1">
+        <v>9.9999999999999995E-8</v>
+      </c>
+      <c r="G22" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H22" s="1">
+        <v>9.9999999999999995E-8</v>
+      </c>
+      <c r="I22" s="1">
+        <v>1.2137458E+19</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B23" s="1">
+        <v>1.9999999999999999E-7</v>
+      </c>
+      <c r="C23" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D23" s="1">
+        <v>1.9999999999999999E-7</v>
+      </c>
+      <c r="E23" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F23" s="1">
+        <v>1.9999999999999999E-7</v>
+      </c>
+      <c r="G23" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H23" s="1">
+        <v>1.9999999999999999E-7</v>
+      </c>
+      <c r="I23" s="1">
+        <v>1.2137458E+19</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B24" s="1">
+        <v>4.2019572E-7</v>
+      </c>
+      <c r="C24" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D24" s="1">
+        <v>4.2019572E-7</v>
+      </c>
+      <c r="E24" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F24" s="1">
+        <v>4.2019572E-7</v>
+      </c>
+      <c r="G24" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H24" s="1">
+        <v>4.2019572E-7</v>
+      </c>
+      <c r="I24" s="1">
+        <v>1.2137457E+19</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B25" s="1">
+        <v>8.6058715000000004E-7</v>
+      </c>
+      <c r="C25" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D25" s="1">
+        <v>8.6058715000000004E-7</v>
+      </c>
+      <c r="E25" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F25" s="1">
+        <v>8.6058715000000004E-7</v>
+      </c>
+      <c r="G25" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H25" s="1">
+        <v>8.6058715000000004E-7</v>
+      </c>
+      <c r="I25" s="1">
+        <v>1.2137454E+19</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B26" s="1">
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="C26" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D26" s="1">
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="E26" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F26" s="1">
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="G26" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H26" s="1">
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="I26" s="1">
+        <v>1.2137454E+19</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B27" s="1">
+        <v>1.8807829000000001E-6</v>
+      </c>
+      <c r="C27" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D27" s="1">
+        <v>1.8807829000000001E-6</v>
+      </c>
+      <c r="E27" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F27" s="1">
+        <v>1.8807829000000001E-6</v>
+      </c>
+      <c r="G27" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="H27" s="1">
+        <v>1.8807829000000001E-6</v>
+      </c>
+      <c r="I27" s="1">
+        <v>1.2137449E+19</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B28" s="1">
+        <v>3.6423486E-6</v>
+      </c>
+      <c r="C28" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D28" s="1">
+        <v>3.6423486E-6</v>
+      </c>
+      <c r="E28" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F28" s="1">
+        <v>3.6423486E-6</v>
+      </c>
+      <c r="G28" s="1">
+        <v>1.1953783E+19</v>
+      </c>
+      <c r="H28" s="1">
+        <v>3.6423486E-6</v>
+      </c>
+      <c r="I28" s="1">
+        <v>1.213744E+19</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B29" s="1">
+        <v>7.1654800999999996E-6</v>
+      </c>
+      <c r="C29" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D29" s="1">
+        <v>7.1654800999999996E-6</v>
+      </c>
+      <c r="E29" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F29" s="1">
+        <v>7.1654800999999996E-6</v>
+      </c>
+      <c r="G29" s="1">
+        <v>1.1953783E+19</v>
+      </c>
+      <c r="H29" s="1">
+        <v>7.1654800999999996E-6</v>
+      </c>
+      <c r="I29" s="1">
+        <v>1.2137422E+19</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B30" s="1">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="C30" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D30" s="1">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="E30" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F30" s="1">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="G30" s="1">
+        <v>1.1953783E+19</v>
+      </c>
+      <c r="H30" s="1">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="I30" s="1">
+        <v>1.2137407E+19</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B31" s="1">
+        <v>1.7046262999999999E-5</v>
+      </c>
+      <c r="C31" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D31" s="1">
+        <v>1.7046262999999999E-5</v>
+      </c>
+      <c r="E31" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F31" s="1">
+        <v>1.7046262999999999E-5</v>
+      </c>
+      <c r="G31" s="1">
+        <v>1.1953783E+19</v>
+      </c>
+      <c r="H31" s="1">
+        <v>1.7046262999999999E-5</v>
+      </c>
+      <c r="I31" s="1">
+        <v>1.213737E+19</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B32" s="1">
+        <v>3.1138788999999997E-5</v>
+      </c>
+      <c r="C32" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D32" s="1">
+        <v>3.1138788999999997E-5</v>
+      </c>
+      <c r="E32" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F32" s="1">
+        <v>3.1138788999999997E-5</v>
+      </c>
+      <c r="G32" s="1">
+        <v>1.1953782E+19</v>
+      </c>
+      <c r="H32" s="1">
+        <v>3.1138788999999997E-5</v>
+      </c>
+      <c r="I32" s="1">
+        <v>1.2137298E+19</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B33" s="1">
+        <v>5.9323841000000002E-5</v>
+      </c>
+      <c r="C33" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D33" s="1">
+        <v>5.9323841000000002E-5</v>
+      </c>
+      <c r="E33" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F33" s="1">
+        <v>5.9323841000000002E-5</v>
+      </c>
+      <c r="G33" s="1">
+        <v>1.195378E+19</v>
+      </c>
+      <c r="H33" s="1">
+        <v>5.9323841000000002E-5</v>
+      </c>
+      <c r="I33" s="1">
+        <v>1.2137155E+19</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B34">
+        <v>1E-4</v>
+      </c>
+      <c r="C34" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D34">
+        <v>1E-4</v>
+      </c>
+      <c r="E34" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F34">
+        <v>1E-4</v>
+      </c>
+      <c r="G34" s="1">
+        <v>1.1953777E+19</v>
+      </c>
+      <c r="H34">
+        <v>1E-4</v>
+      </c>
+      <c r="I34" s="1">
+        <v>1.2136952E+19</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B35">
+        <v>2.1274021E-4</v>
+      </c>
+      <c r="C35" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D35">
+        <v>2.1274021E-4</v>
+      </c>
+      <c r="E35" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F35">
+        <v>2.1274021E-4</v>
+      </c>
+      <c r="G35" s="1">
+        <v>1.195377E+19</v>
+      </c>
+      <c r="H35">
+        <v>2.1274021E-4</v>
+      </c>
+      <c r="I35" s="1">
+        <v>1.2136416E+19</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B36">
+        <v>4.3822061999999998E-4</v>
+      </c>
+      <c r="C36" s="1">
+        <v>1.1050604E+19</v>
+      </c>
+      <c r="D36">
+        <v>4.3822061999999998E-4</v>
+      </c>
+      <c r="E36" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F36">
+        <v>4.3822061999999998E-4</v>
+      </c>
+      <c r="G36" s="1">
+        <v>1.1953756E+19</v>
+      </c>
+      <c r="H36">
+        <v>4.3822061999999998E-4</v>
+      </c>
+      <c r="I36" s="1">
+        <v>1.2135427E+19</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B37">
+        <v>8.8918145E-4</v>
+      </c>
+      <c r="C37" s="1">
+        <v>1.1050603E+19</v>
+      </c>
+      <c r="D37">
+        <v>8.8918145E-4</v>
+      </c>
+      <c r="E37" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F37">
+        <v>8.8918145E-4</v>
+      </c>
+      <c r="G37" s="1">
+        <v>1.1953729E+19</v>
+      </c>
+      <c r="H37">
+        <v>8.8918145E-4</v>
+      </c>
+      <c r="I37" s="1">
+        <v>1.2133695E+19</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B38">
+        <v>1E-3</v>
+      </c>
+      <c r="C38" s="1">
+        <v>1.1050603E+19</v>
+      </c>
+      <c r="D38">
+        <v>1E-3</v>
+      </c>
+      <c r="E38" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F38">
+        <v>1E-3</v>
+      </c>
+      <c r="G38" s="1">
+        <v>1.1953722E+19</v>
+      </c>
+      <c r="H38">
+        <v>1E-3</v>
+      </c>
+      <c r="I38" s="1">
+        <v>1.2133283E+19</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B39">
+        <v>1.9019217E-3</v>
+      </c>
+      <c r="C39" s="1">
+        <v>1.1050603E+19</v>
+      </c>
+      <c r="D39">
+        <v>1.9019217E-3</v>
+      </c>
+      <c r="E39" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F39">
+        <v>1.9019217E-3</v>
+      </c>
+      <c r="G39" s="1">
+        <v>1.1953666E+19</v>
+      </c>
+      <c r="H39">
+        <v>1.9019217E-3</v>
+      </c>
+      <c r="I39" s="1">
+        <v>1.2130518E+19</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B40">
+        <v>3.7057650000000002E-3</v>
+      </c>
+      <c r="C40" s="1">
+        <v>1.1050601E+19</v>
+      </c>
+      <c r="D40">
+        <v>3.7057650000000002E-3</v>
+      </c>
+      <c r="E40" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F40">
+        <v>3.7057650000000002E-3</v>
+      </c>
+      <c r="G40" s="1">
+        <v>1.1953558E+19</v>
+      </c>
+      <c r="H40">
+        <v>3.7057650000000002E-3</v>
+      </c>
+      <c r="I40" s="1">
+        <v>1.2126289E+19</v>
+      </c>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B41">
+        <v>7.3134515999999997E-3</v>
+      </c>
+      <c r="C41" s="1">
+        <v>1.1050599E+19</v>
+      </c>
+      <c r="D41">
+        <v>7.3134515999999997E-3</v>
+      </c>
+      <c r="E41" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F41">
+        <v>7.3134515999999997E-3</v>
+      </c>
+      <c r="G41" s="1">
+        <v>1.1953346E+19</v>
+      </c>
+      <c r="H41">
+        <v>7.3134515999999997E-3</v>
+      </c>
+      <c r="I41" s="1">
+        <v>1.2120324E+19</v>
+      </c>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B42">
+        <v>0.01</v>
+      </c>
+      <c r="C42" s="1">
+        <v>1.1050596E+19</v>
+      </c>
+      <c r="D42">
+        <v>0.01</v>
+      </c>
+      <c r="E42" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F42">
+        <v>0.01</v>
+      </c>
+      <c r="G42" s="1">
+        <v>1.1953191E+19</v>
+      </c>
+      <c r="H42">
+        <v>0.01</v>
+      </c>
+      <c r="I42" s="1">
+        <v>1.2116741E+19</v>
+      </c>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B43">
+        <v>1.7215372999999999E-2</v>
+      </c>
+      <c r="C43" s="1">
+        <v>1.1050591E+19</v>
+      </c>
+      <c r="D43">
+        <v>1.7215372999999999E-2</v>
+      </c>
+      <c r="E43" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F43">
+        <v>1.7215372999999999E-2</v>
+      </c>
+      <c r="G43" s="1">
+        <v>1.1952797E+19</v>
+      </c>
+      <c r="H43">
+        <v>1.7215372999999999E-2</v>
+      </c>
+      <c r="I43" s="1">
+        <v>1.2110071E+19</v>
+      </c>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B44">
+        <v>3.164612E-2</v>
+      </c>
+      <c r="C44" s="1">
+        <v>1.105058E+19</v>
+      </c>
+      <c r="D44">
+        <v>3.164612E-2</v>
+      </c>
+      <c r="E44" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F44">
+        <v>3.164612E-2</v>
+      </c>
+      <c r="G44" s="1">
+        <v>1.1952073E+19</v>
+      </c>
+      <c r="H44">
+        <v>3.164612E-2</v>
+      </c>
+      <c r="I44" s="1">
+        <v>1.2101588E+19</v>
+      </c>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B45">
+        <v>6.0507613000000002E-2</v>
+      </c>
+      <c r="C45" s="1">
+        <v>1.1050558E+19</v>
+      </c>
+      <c r="D45">
+        <v>6.0507613000000002E-2</v>
+      </c>
+      <c r="E45" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F45">
+        <v>6.0507613000000002E-2</v>
+      </c>
+      <c r="G45" s="1">
+        <v>1.195081E+19</v>
+      </c>
+      <c r="H45">
+        <v>6.0507613000000002E-2</v>
+      </c>
+      <c r="I45" s="1">
+        <v>1.20916E+19</v>
+      </c>
+    </row>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B46">
+        <v>0.1</v>
+      </c>
+      <c r="C46" s="1">
+        <v>1.1050528E+19</v>
+      </c>
+      <c r="D46">
+        <v>0.1</v>
+      </c>
+      <c r="E46" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F46">
+        <v>0.1</v>
+      </c>
+      <c r="G46" s="1">
+        <v>1.194932E+19</v>
+      </c>
+      <c r="H46">
+        <v>0.1</v>
+      </c>
+      <c r="I46" s="1">
+        <v>1.208306E+19</v>
+      </c>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B47">
+        <v>0.2</v>
+      </c>
+      <c r="C47" s="1">
+        <v>1.1050453E+19</v>
+      </c>
+      <c r="D47">
+        <v>0.2</v>
+      </c>
+      <c r="E47" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F47">
+        <v>0.2</v>
+      </c>
+      <c r="G47" s="1">
+        <v>1.1946388E+19</v>
+      </c>
+      <c r="H47">
+        <v>0.2</v>
+      </c>
+      <c r="I47" s="1">
+        <v>1.2071348E+19</v>
+      </c>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B48">
+        <v>0.43089195000000002</v>
+      </c>
+      <c r="C48" s="1">
+        <v>1.1050287E+19</v>
+      </c>
+      <c r="D48">
+        <v>0.43089195000000002</v>
+      </c>
+      <c r="E48" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F48">
+        <v>0.43089195000000002</v>
+      </c>
+      <c r="G48" s="1">
+        <v>1.1941634E+19</v>
+      </c>
+      <c r="H48">
+        <v>0.43089195000000002</v>
+      </c>
+      <c r="I48" s="1">
+        <v>1.2057637E+19</v>
+      </c>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B49">
+        <v>0.5</v>
+      </c>
+      <c r="C49" s="1">
+        <v>1.1050238E+19</v>
+      </c>
+      <c r="D49">
+        <v>0.5</v>
+      </c>
+      <c r="E49" s="1">
+        <v>9.1386937E+18</v>
+      </c>
+      <c r="F49">
+        <v>0.5</v>
+      </c>
+      <c r="G49" s="1">
+        <v>1.1940351E+19</v>
+      </c>
+      <c r="H49">
+        <v>0.5</v>
+      </c>
+      <c r="I49" s="1">
+        <v>1.2054261E+19</v>
+      </c>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B50">
+        <v>0.96178388999999997</v>
+      </c>
+      <c r="C50" s="1">
+        <v>1.104993E+19</v>
+      </c>
+      <c r="D50">
+        <v>0.96178388999999997</v>
+      </c>
+      <c r="E50" s="1">
+        <v>9.1386936E+18</v>
+      </c>
+      <c r="F50">
+        <v>0.96178388999999997</v>
+      </c>
+      <c r="G50" s="1">
+        <v>1.1934505E+19</v>
+      </c>
+      <c r="H50">
+        <v>0.96178388999999997</v>
+      </c>
+      <c r="I50" s="1">
+        <v>1.2041111E+19</v>
+      </c>
+    </row>
+    <row r="51" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B51">
+        <v>1</v>
+      </c>
+      <c r="C51" s="1">
+        <v>1.1049904E+19</v>
+      </c>
+      <c r="D51">
+        <v>1</v>
+      </c>
+      <c r="E51" s="1">
+        <v>9.1386936E+18</v>
+      </c>
+      <c r="F51">
+        <v>1</v>
+      </c>
+      <c r="G51" s="1">
+        <v>1.1934038E+19</v>
+      </c>
+      <c r="H51">
+        <v>1</v>
+      </c>
+      <c r="I51" s="1">
+        <v>1.2040077E+19</v>
+      </c>
+    </row>
+    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B52">
+        <v>1.9235678</v>
+      </c>
+      <c r="C52" s="1">
+        <v>1.1049351E+19</v>
+      </c>
+      <c r="D52">
+        <v>1.4617838999999999</v>
+      </c>
+      <c r="E52" s="1">
+        <v>9.1386936E+18</v>
+      </c>
+      <c r="F52">
+        <v>1.9235678</v>
+      </c>
+      <c r="G52" s="1">
+        <v>1.1926787E+19</v>
+      </c>
+      <c r="H52">
+        <v>1.9235678</v>
+      </c>
+      <c r="I52" s="1">
+        <v>1.2024379E+19</v>
+      </c>
+    </row>
+    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B53">
+        <v>2</v>
+      </c>
+      <c r="C53" s="1">
+        <v>1.1049306E+19</v>
+      </c>
+      <c r="D53">
+        <v>2</v>
+      </c>
+      <c r="E53" s="1">
+        <v>9.1386935E+18</v>
+      </c>
+      <c r="F53">
+        <v>2</v>
+      </c>
+      <c r="G53" s="1">
+        <v>1.1926211E+19</v>
+      </c>
+      <c r="H53">
+        <v>2</v>
+      </c>
+      <c r="I53" s="1">
+        <v>1.2023133E+19</v>
+      </c>
+    </row>
+    <row r="54" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B54">
+        <v>2.4617838999999999</v>
+      </c>
+      <c r="C54" s="1">
+        <v>1.1049044E+19</v>
+      </c>
+      <c r="D54">
+        <v>2.8509943999999998</v>
+      </c>
+      <c r="E54" s="1">
+        <v>9.1386934E+18</v>
+      </c>
+      <c r="F54">
+        <v>2.4617838999999999</v>
+      </c>
+      <c r="G54" s="1">
+        <v>1.1923333E+19</v>
+      </c>
+      <c r="H54">
+        <v>3.8471356000000001</v>
+      </c>
+      <c r="I54" s="1">
+        <v>1.2002551E+19</v>
+      </c>
+    </row>
+    <row r="55" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B55">
+        <v>2.9235677999999998</v>
+      </c>
+      <c r="C55" s="1">
+        <v>1.1048794E+19</v>
+      </c>
+      <c r="D55">
+        <v>3.4254972000000001</v>
+      </c>
+      <c r="E55" s="1">
+        <v>9.1386933E+18</v>
+      </c>
+      <c r="F55">
+        <v>3.3853517000000002</v>
+      </c>
+      <c r="G55" s="1">
+        <v>1.191894E+19</v>
+      </c>
+      <c r="H55">
+        <v>4</v>
+      </c>
+      <c r="I55" s="1">
+        <v>1.2000904E+19</v>
+      </c>
+    </row>
+    <row r="56" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B56">
+        <v>3.8471356000000001</v>
+      </c>
+      <c r="C56" s="1">
+        <v>1.104833E+19</v>
+      </c>
+      <c r="D56">
+        <v>4</v>
+      </c>
+      <c r="E56" s="1">
+        <v>9.1386932E+18</v>
+      </c>
+      <c r="F56">
+        <v>4</v>
+      </c>
+      <c r="G56" s="1">
+        <v>1.1916446E+19</v>
+      </c>
+      <c r="H56">
+        <v>4.9235677999999998</v>
+      </c>
+      <c r="I56" s="1">
+        <v>1.1992176E+19</v>
+      </c>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B57">
+        <v>4</v>
+      </c>
+      <c r="C57" s="1">
+        <v>1.1048254E+19</v>
+      </c>
+      <c r="D57">
+        <v>5.8167374000000001</v>
+      </c>
+      <c r="E57" s="1">
+        <v>9.138693E+18</v>
+      </c>
+      <c r="F57">
+        <v>4.9235677999999998</v>
+      </c>
+      <c r="G57" s="1">
+        <v>1.1913349E+19</v>
+      </c>
+      <c r="H57">
+        <v>5.8471355999999997</v>
+      </c>
+      <c r="I57" s="1">
+        <v>1.1984281E+19</v>
+      </c>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B58">
+        <v>4.9235677999999998</v>
+      </c>
+      <c r="C58" s="1">
+        <v>1.1047825E+19</v>
+      </c>
+      <c r="D58">
+        <v>6.9083686999999996</v>
+      </c>
+      <c r="E58" s="1">
+        <v>9.1386929E+18</v>
+      </c>
+      <c r="F58">
+        <v>5.3853517000000002</v>
+      </c>
+      <c r="G58" s="1">
+        <v>1.1911935E+19</v>
+      </c>
+      <c r="H58">
+        <v>7.6942710999999999</v>
+      </c>
+      <c r="I58" s="1">
+        <v>1.1970581E+19</v>
+      </c>
+    </row>
+    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B59">
+        <v>6.7707033000000001</v>
+      </c>
+      <c r="C59" s="1">
+        <v>1.1047054E+19</v>
+      </c>
+      <c r="D59">
+        <v>8</v>
+      </c>
+      <c r="E59" s="1">
+        <v>9.1386927E+18</v>
+      </c>
+      <c r="F59">
+        <v>6.3089195</v>
+      </c>
+      <c r="G59" s="1">
+        <v>1.1909499E+19</v>
+      </c>
+      <c r="H59">
+        <v>8</v>
+      </c>
+      <c r="I59" s="1">
+        <v>1.1968366E+19</v>
+      </c>
+    </row>
+    <row r="60" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B60">
+        <v>8</v>
+      </c>
+      <c r="C60" s="1">
+        <v>1.1046573E+19</v>
+      </c>
+      <c r="D60">
+        <v>9.0916312999999995</v>
+      </c>
+      <c r="E60" s="1">
+        <v>9.1386926E+18</v>
+      </c>
+      <c r="F60">
+        <v>8</v>
+      </c>
+      <c r="G60" s="1">
+        <v>1.19059E+19</v>
+      </c>
+      <c r="H60">
+        <v>11.694271000000001</v>
+      </c>
+      <c r="I60" s="1">
+        <v>1.1946294E+19</v>
+      </c>
+    </row>
+    <row r="61" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B61">
+        <v>9.8471355999999997</v>
+      </c>
+      <c r="C61" s="1">
+        <v>1.1045909E+19</v>
+      </c>
+      <c r="D61">
+        <v>9.6374469999999999</v>
+      </c>
+      <c r="E61" s="1">
+        <v>9.1386925E+18</v>
+      </c>
+      <c r="F61">
+        <v>11.694271000000001</v>
+      </c>
+      <c r="G61" s="1">
+        <v>1.1900226E+19</v>
+      </c>
+      <c r="H61">
+        <v>12.770702999999999</v>
+      </c>
+      <c r="I61" s="1">
+        <v>1.1940209E+19</v>
+      </c>
+    </row>
+    <row r="62" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B62">
+        <v>10.770702999999999</v>
+      </c>
+      <c r="C62" s="1">
+        <v>1.104559E+19</v>
+      </c>
+      <c r="D62">
+        <v>10.183263</v>
+      </c>
+      <c r="E62" s="1">
+        <v>9.1386925E+18</v>
+      </c>
+      <c r="F62">
+        <v>12.770702999999999</v>
+      </c>
+      <c r="G62" s="1">
+        <v>1.1898724E+19</v>
+      </c>
+      <c r="H62">
+        <v>14.923568</v>
+      </c>
+      <c r="I62" s="1">
+        <v>1.1929154E+19</v>
+      </c>
+    </row>
+    <row r="63" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B63">
+        <v>11.694271000000001</v>
+      </c>
+      <c r="C63" s="1">
+        <v>1.1045282E+19</v>
+      </c>
+      <c r="D63">
+        <v>10.729077999999999</v>
+      </c>
+      <c r="E63" s="1">
+        <v>9.1386924E+18</v>
+      </c>
+      <c r="F63">
+        <v>13.308918999999999</v>
+      </c>
+      <c r="G63" s="1">
+        <v>1.1898008E+19</v>
+      </c>
+      <c r="H63">
+        <v>16</v>
+      </c>
+      <c r="I63" s="1">
+        <v>1.192388E+19</v>
+      </c>
+    </row>
+    <row r="64" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B64">
+        <v>13.541407</v>
+      </c>
+      <c r="C64" s="1">
+        <v>1.1044707E+19</v>
+      </c>
+      <c r="D64">
+        <v>11.274894</v>
+      </c>
+      <c r="E64" s="1">
+        <v>9.1386923E+18</v>
+      </c>
+      <c r="F64">
+        <v>14.385351999999999</v>
+      </c>
+      <c r="G64" s="1">
+        <v>1.189669E+19</v>
+      </c>
+      <c r="H64">
+        <v>17.076432</v>
+      </c>
+      <c r="I64" s="1">
+        <v>1.1918836E+19</v>
+      </c>
+    </row>
+    <row r="65" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B65">
+        <v>14.770702999999999</v>
+      </c>
+      <c r="C65" s="1">
+        <v>1.104434E+19</v>
+      </c>
+      <c r="D65">
+        <v>11.82071</v>
+      </c>
+      <c r="E65" s="1">
+        <v>9.1386923E+18</v>
+      </c>
+      <c r="F65">
+        <v>15.192676000000001</v>
+      </c>
+      <c r="G65" s="1">
+        <v>1.1895759E+19</v>
+      </c>
+      <c r="H65">
+        <v>19.229296999999999</v>
+      </c>
+      <c r="I65" s="1">
+        <v>1.1909537E+19</v>
+      </c>
+    </row>
+    <row r="66" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B66">
+        <v>16</v>
+      </c>
+      <c r="C66" s="1">
+        <v>1.1043987E+19</v>
+      </c>
+      <c r="D66">
+        <v>12.366524999999999</v>
+      </c>
+      <c r="E66" s="1">
+        <v>9.1386922E+18</v>
+      </c>
+      <c r="F66">
+        <v>16</v>
+      </c>
+      <c r="G66" s="1">
+        <v>1.1894878E+19</v>
+      </c>
+      <c r="H66">
+        <v>21.382161</v>
+      </c>
+      <c r="I66" s="1">
+        <v>1.1900924E+19</v>
+      </c>
+    </row>
+    <row r="67" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B67" t="s">
+        <v>14</v>
+      </c>
+      <c r="C67" t="s">
+        <v>14</v>
+      </c>
+      <c r="D67">
+        <v>13.458157</v>
+      </c>
+      <c r="E67" s="1">
+        <v>9.1386921E+18</v>
+      </c>
+      <c r="F67">
+        <v>18.552983000000001</v>
+      </c>
+      <c r="G67" s="1">
+        <v>1.1892472E+19</v>
+      </c>
+      <c r="H67">
+        <v>22.458593</v>
+      </c>
+      <c r="I67" s="1">
+        <v>1.1896778E+19</v>
+      </c>
+    </row>
+    <row r="68" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B68" t="s">
+        <v>14</v>
+      </c>
+      <c r="C68" t="s">
+        <v>14</v>
+      </c>
+      <c r="D68">
+        <v>14.003971999999999</v>
+      </c>
+      <c r="E68" s="1">
+        <v>9.138692E+18</v>
+      </c>
+      <c r="F68">
+        <v>19.191229</v>
+      </c>
+      <c r="G68" s="1">
+        <v>1.1891893E+19</v>
+      </c>
+      <c r="H68">
+        <v>22.996808999999999</v>
+      </c>
+      <c r="I68" s="1">
+        <v>1.1894743E+19</v>
+      </c>
+    </row>
+    <row r="69" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B69" t="s">
+        <v>14</v>
+      </c>
+      <c r="C69" t="s">
+        <v>14</v>
+      </c>
+      <c r="D69">
+        <v>14.549787999999999</v>
+      </c>
+      <c r="E69" s="1">
+        <v>9.1386919E+18</v>
+      </c>
+      <c r="F69">
+        <v>19.829474999999999</v>
+      </c>
+      <c r="G69" s="1">
+        <v>1.1891333E+19</v>
+      </c>
+      <c r="H69">
+        <v>24.073242</v>
+      </c>
+      <c r="I69" s="1">
+        <v>1.1890818E+19</v>
+      </c>
+    </row>
+    <row r="70" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B70" t="s">
+        <v>14</v>
+      </c>
+      <c r="C70" t="s">
+        <v>14</v>
+      </c>
+      <c r="D70">
+        <v>15.095603000000001</v>
+      </c>
+      <c r="E70" s="1">
+        <v>9.1386919E+18</v>
+      </c>
+      <c r="F70">
+        <v>21.105965999999999</v>
+      </c>
+      <c r="G70" s="1">
+        <v>1.1890285E+19</v>
+      </c>
+      <c r="H70">
+        <v>25.149674000000001</v>
+      </c>
+      <c r="I70" s="1">
+        <v>1.188703E+19</v>
+      </c>
+    </row>
+    <row r="71" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B71" t="s">
+        <v>14</v>
+      </c>
+      <c r="C71" t="s">
+        <v>14</v>
+      </c>
+      <c r="D71">
+        <v>16</v>
+      </c>
+      <c r="E71" s="1">
+        <v>9.1386918E+18</v>
+      </c>
+      <c r="F71">
+        <v>22.382458</v>
+      </c>
+      <c r="G71" s="1">
+        <v>1.18893E+19</v>
+      </c>
+      <c r="H71">
+        <v>26.226106000000001</v>
+      </c>
+      <c r="I71" s="1">
+        <v>1.188337E+19</v>
+      </c>
+    </row>
+    <row r="72" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B72" t="s">
+        <v>14</v>
+      </c>
+      <c r="C72" t="s">
+        <v>14</v>
+      </c>
+      <c r="D72">
+        <v>16.545815999999999</v>
+      </c>
+      <c r="E72" s="1">
+        <v>9.1386917E+18</v>
+      </c>
+      <c r="F72" t="s">
+        <v>14</v>
+      </c>
+      <c r="G72" t="s">
+        <v>14</v>
+      </c>
+      <c r="H72">
+        <v>26.764322</v>
+      </c>
+      <c r="I72" s="1">
+        <v>1.1881571E+19</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61E7C826-F786-4EE7-9C76-F06B5176B29E}">
   <dimension ref="A1:R47"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -6088,7 +7934,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C4C1E0D-2AEE-4A7F-82EA-F9A1189D6A82}">
   <dimension ref="A1:K1050"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -18354,7 +20200,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0971B89F-4BB2-40B3-A650-BC46BAF40E7C}">
   <dimension ref="A1:P162"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Figure change, but manuscript must be done later. 감기걸려서 죽을맛이다
</commit_message>
<xml_diff>
--- a/figures/TCAD data.xlsx
+++ b/figures/TCAD data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshs\Desktop\local-laptop\EDLtarget-manuscript-December\figures\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshs\Desktop\GitUpload\EDLtarget-manuscript-Jan\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEA71504-E459-4B0E-B22C-324A39F91EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC28197-49AB-40DB-8D85-66A58BCA25BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6E1D205E-5548-4B10-8EA6-16E0E10C324F}"/>
+    <workbookView xWindow="18225" yWindow="4740" windowWidth="18870" windowHeight="11370" activeTab="1" xr2:uid="{6E1D205E-5548-4B10-8EA6-16E0E10C324F}"/>
   </bookViews>
   <sheets>
     <sheet name="1 V pgm 300-125-cryogenic raw" sheetId="4" r:id="rId1"/>
@@ -3818,24 +3818,27 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB8F665F-4B87-445E-8D0D-37A1126372C0}">
-  <dimension ref="B2:I72"/>
+  <dimension ref="B2:M72"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="9.25" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="E2" t="s">
         <v>0</v>
       </c>
       <c r="H2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="K2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B3" s="1">
         <v>9.9999999999999998E-13</v>
       </c>
@@ -3843,25 +3846,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D3" s="1">
+        <f>12100000000000000000-C$3+C3</f>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E3" s="1">
         <v>9.9999999999999998E-13</v>
       </c>
-      <c r="E3" s="1">
+      <c r="F3" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F3" s="1">
-        <v>9.9999999999999998E-13</v>
-      </c>
       <c r="G3" s="1">
-        <v>1.1953784E+19</v>
+        <f>12100000000000000000-F$3+F3</f>
+        <v>1.21E+19</v>
       </c>
       <c r="H3" s="1">
         <v>9.9999999999999998E-13</v>
       </c>
       <c r="I3" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J3" s="1">
+        <f>12100000000000000000-I$3+I3</f>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K3" s="1">
+        <v>9.9999999999999998E-13</v>
+      </c>
+      <c r="L3" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M3" s="1">
+        <f>12100000000000000000-L$3+L3</f>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="4" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B4" s="1">
         <v>3.0000000000000001E-12</v>
       </c>
@@ -3869,25 +3888,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D4" s="1">
+        <f t="shared" ref="D4:D67" si="0">12100000000000000000-C$3+C4</f>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E4" s="1">
         <v>3.0000000000000001E-12</v>
       </c>
-      <c r="E4" s="1">
+      <c r="F4" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F4" s="1">
-        <v>3.0000000000000001E-12</v>
-      </c>
       <c r="G4" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" ref="G4:G67" si="1">12100000000000000000-F$3+F4</f>
+        <v>1.21E+19</v>
       </c>
       <c r="H4" s="1">
         <v>3.0000000000000001E-12</v>
       </c>
       <c r="I4" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J4" s="1">
+        <f t="shared" ref="J4:J67" si="2">12100000000000000000-I$3+I4</f>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K4" s="1">
+        <v>3.0000000000000001E-12</v>
+      </c>
+      <c r="L4" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M4" s="1">
+        <f t="shared" ref="M4:M67" si="3">12100000000000000000-L$3+L4</f>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B5" s="1">
         <v>7.0000000000000001E-12</v>
       </c>
@@ -3895,25 +3930,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D5" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E5" s="1">
         <v>7.0000000000000001E-12</v>
       </c>
-      <c r="E5" s="1">
+      <c r="F5" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F5" s="1">
-        <v>7.0000000000000001E-12</v>
-      </c>
       <c r="G5" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H5" s="1">
         <v>7.0000000000000001E-12</v>
       </c>
       <c r="I5" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J5" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K5" s="1">
+        <v>7.0000000000000001E-12</v>
+      </c>
+      <c r="L5" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M5" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B6" s="1">
         <v>9.9999999999999994E-12</v>
       </c>
@@ -3921,25 +3972,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D6" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E6" s="1">
         <v>9.9999999999999994E-12</v>
       </c>
-      <c r="E6" s="1">
+      <c r="F6" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F6" s="1">
-        <v>9.9999999999999994E-12</v>
-      </c>
       <c r="G6" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H6" s="1">
         <v>9.9999999999999994E-12</v>
       </c>
       <c r="I6" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J6" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K6" s="1">
+        <v>9.9999999999999994E-12</v>
+      </c>
+      <c r="L6" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M6" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B7" s="1">
         <v>1.7999999999999999E-11</v>
       </c>
@@ -3947,25 +4014,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D7" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E7" s="1">
         <v>1.7999999999999999E-11</v>
       </c>
-      <c r="E7" s="1">
+      <c r="F7" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F7" s="1">
-        <v>1.7999999999999999E-11</v>
-      </c>
       <c r="G7" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H7" s="1">
         <v>1.7999999999999999E-11</v>
       </c>
       <c r="I7" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J7" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K7" s="1">
+        <v>1.7999999999999999E-11</v>
+      </c>
+      <c r="L7" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M7" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B8" s="1">
         <v>3.3999999999999999E-11</v>
       </c>
@@ -3973,25 +4056,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D8" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E8" s="1">
         <v>3.3999999999999999E-11</v>
       </c>
-      <c r="E8" s="1">
+      <c r="F8" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F8" s="1">
-        <v>3.3999999999999999E-11</v>
-      </c>
       <c r="G8" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H8" s="1">
         <v>3.3999999999999999E-11</v>
       </c>
       <c r="I8" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J8" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K8" s="1">
+        <v>3.3999999999999999E-11</v>
+      </c>
+      <c r="L8" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M8" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B9" s="1">
         <v>6.6000000000000005E-11</v>
       </c>
@@ -3999,25 +4098,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D9" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E9" s="1">
         <v>6.6000000000000005E-11</v>
       </c>
-      <c r="E9" s="1">
+      <c r="F9" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F9" s="1">
-        <v>6.6000000000000005E-11</v>
-      </c>
       <c r="G9" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H9" s="1">
         <v>6.6000000000000005E-11</v>
       </c>
       <c r="I9" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J9" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K9" s="1">
+        <v>6.6000000000000005E-11</v>
+      </c>
+      <c r="L9" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M9" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B10" s="1">
         <v>1E-10</v>
       </c>
@@ -4025,25 +4140,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D10" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E10" s="1">
         <v>1E-10</v>
       </c>
-      <c r="E10" s="1">
+      <c r="F10" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F10" s="1">
-        <v>1E-10</v>
-      </c>
       <c r="G10" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H10" s="1">
         <v>1E-10</v>
       </c>
       <c r="I10" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J10" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K10" s="1">
+        <v>1E-10</v>
+      </c>
+      <c r="L10" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M10" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B11" s="1">
         <v>2.0751743999999999E-10</v>
       </c>
@@ -4051,25 +4182,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D11" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E11" s="1">
         <v>2.0751743999999999E-10</v>
       </c>
-      <c r="E11" s="1">
+      <c r="F11" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F11" s="1">
-        <v>2.0751743999999999E-10</v>
-      </c>
       <c r="G11" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H11" s="1">
         <v>2.0751743999999999E-10</v>
       </c>
       <c r="I11" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J11" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K11" s="1">
+        <v>2.0751743999999999E-10</v>
+      </c>
+      <c r="L11" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M11" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B12" s="1">
         <v>4.2255232E-10</v>
       </c>
@@ -4077,25 +4224,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D12" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E12" s="1">
         <v>4.2255232E-10</v>
       </c>
-      <c r="E12" s="1">
+      <c r="F12" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F12" s="1">
-        <v>4.2255232E-10</v>
-      </c>
       <c r="G12" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H12" s="1">
         <v>4.2255232E-10</v>
       </c>
       <c r="I12" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J12" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K12" s="1">
+        <v>4.2255232E-10</v>
+      </c>
+      <c r="L12" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M12" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B13" s="1">
         <v>8.5262207999999996E-10</v>
       </c>
@@ -4103,25 +4266,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D13" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E13" s="1">
         <v>8.5262207999999996E-10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="F13" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F13" s="1">
-        <v>8.5262207999999996E-10</v>
-      </c>
       <c r="G13" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H13" s="1">
         <v>8.5262207999999996E-10</v>
       </c>
       <c r="I13" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J13" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K13" s="1">
+        <v>8.5262207999999996E-10</v>
+      </c>
+      <c r="L13" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M13" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B14" s="1">
         <v>1.0000000000000001E-9</v>
       </c>
@@ -4129,25 +4308,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D14" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E14" s="1">
         <v>1.0000000000000001E-9</v>
       </c>
-      <c r="E14" s="1">
+      <c r="F14" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F14" s="1">
-        <v>1.0000000000000001E-9</v>
-      </c>
       <c r="G14" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H14" s="1">
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="I14" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J14" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K14" s="1">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="L14" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M14" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="15" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B15" s="1">
         <v>1.8601395E-9</v>
       </c>
@@ -4155,25 +4350,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D15" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E15" s="1">
         <v>1.8601395E-9</v>
       </c>
-      <c r="E15" s="1">
+      <c r="F15" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F15" s="1">
-        <v>1.8601395E-9</v>
-      </c>
       <c r="G15" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H15" s="1">
         <v>1.8601395E-9</v>
       </c>
       <c r="I15" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J15" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K15" s="1">
+        <v>1.8601395E-9</v>
+      </c>
+      <c r="L15" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M15" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B16" s="1">
         <v>3.5804185999999999E-9</v>
       </c>
@@ -4181,25 +4392,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D16" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E16" s="1">
         <v>3.5804185999999999E-9</v>
       </c>
-      <c r="E16" s="1">
+      <c r="F16" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F16" s="1">
-        <v>3.5804185999999999E-9</v>
-      </c>
       <c r="G16" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H16" s="1">
         <v>3.5804185999999999E-9</v>
       </c>
       <c r="I16" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J16" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K16" s="1">
+        <v>3.5804185999999999E-9</v>
+      </c>
+      <c r="L16" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M16" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B17" s="1">
         <v>7.0209766999999997E-9</v>
       </c>
@@ -4207,25 +4434,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D17" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E17" s="1">
         <v>7.0209766999999997E-9</v>
       </c>
-      <c r="E17" s="1">
+      <c r="F17" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F17" s="1">
-        <v>7.0209766999999997E-9</v>
-      </c>
       <c r="G17" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H17" s="1">
         <v>7.0209766999999997E-9</v>
       </c>
       <c r="I17" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J17" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K17" s="1">
+        <v>7.0209766999999997E-9</v>
+      </c>
+      <c r="L17" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M17" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B18" s="1">
         <v>1E-8</v>
       </c>
@@ -4233,25 +4476,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D18" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E18" s="1">
         <v>1E-8</v>
       </c>
-      <c r="E18" s="1">
+      <c r="F18" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F18" s="1">
-        <v>1E-8</v>
-      </c>
       <c r="G18" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H18" s="1">
         <v>1E-8</v>
       </c>
       <c r="I18" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J18" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K18" s="1">
+        <v>1E-8</v>
+      </c>
+      <c r="L18" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M18" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B19" s="1">
         <v>1.6881116000000001E-8</v>
       </c>
@@ -4259,25 +4518,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D19" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E19" s="1">
         <v>1.6881116000000001E-8</v>
       </c>
-      <c r="E19" s="1">
+      <c r="F19" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F19" s="1">
-        <v>1.6881116000000001E-8</v>
-      </c>
       <c r="G19" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H19" s="1">
         <v>1.6881116000000001E-8</v>
       </c>
       <c r="I19" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J19" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K19" s="1">
+        <v>1.6881116000000001E-8</v>
+      </c>
+      <c r="L19" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M19" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B20" s="1">
         <v>3.0643349000000001E-8</v>
       </c>
@@ -4285,25 +4560,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D20" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E20" s="1">
         <v>3.0643349000000001E-8</v>
       </c>
-      <c r="E20" s="1">
+      <c r="F20" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F20" s="1">
-        <v>3.0643349000000001E-8</v>
-      </c>
       <c r="G20" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H20" s="1">
         <v>3.0643349000000001E-8</v>
       </c>
       <c r="I20" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J20" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K20" s="1">
+        <v>3.0643349000000001E-8</v>
+      </c>
+      <c r="L20" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M20" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B21" s="1">
         <v>5.8167812999999998E-8</v>
       </c>
@@ -4311,25 +4602,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D21" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E21" s="1">
         <v>5.8167812999999998E-8</v>
       </c>
-      <c r="E21" s="1">
+      <c r="F21" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F21" s="1">
-        <v>5.8167812999999998E-8</v>
-      </c>
       <c r="G21" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H21" s="1">
         <v>5.8167812999999998E-8</v>
       </c>
       <c r="I21" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J21" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K21" s="1">
+        <v>5.8167812999999998E-8</v>
+      </c>
+      <c r="L21" s="1">
         <v>1.2137459E+19</v>
       </c>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M21" s="1">
+        <f t="shared" si="3"/>
+        <v>1.21E+19</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B22" s="1">
         <v>9.9999999999999995E-8</v>
       </c>
@@ -4337,25 +4644,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D22" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E22" s="1">
         <v>9.9999999999999995E-8</v>
       </c>
-      <c r="E22" s="1">
+      <c r="F22" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F22" s="1">
-        <v>9.9999999999999995E-8</v>
-      </c>
       <c r="G22" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H22" s="1">
         <v>9.9999999999999995E-8</v>
       </c>
       <c r="I22" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J22" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K22" s="1">
+        <v>9.9999999999999995E-8</v>
+      </c>
+      <c r="L22" s="1">
         <v>1.2137458E+19</v>
       </c>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M22" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2099999E+19</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B23" s="1">
         <v>1.9999999999999999E-7</v>
       </c>
@@ -4363,25 +4686,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D23" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E23" s="1">
         <v>1.9999999999999999E-7</v>
       </c>
-      <c r="E23" s="1">
+      <c r="F23" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F23" s="1">
-        <v>1.9999999999999999E-7</v>
-      </c>
       <c r="G23" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H23" s="1">
         <v>1.9999999999999999E-7</v>
       </c>
       <c r="I23" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J23" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K23" s="1">
+        <v>1.9999999999999999E-7</v>
+      </c>
+      <c r="L23" s="1">
         <v>1.2137458E+19</v>
       </c>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M23" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2099999E+19</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B24" s="1">
         <v>4.2019572E-7</v>
       </c>
@@ -4389,25 +4728,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D24" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E24" s="1">
         <v>4.2019572E-7</v>
       </c>
-      <c r="E24" s="1">
+      <c r="F24" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F24" s="1">
-        <v>4.2019572E-7</v>
-      </c>
       <c r="G24" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H24" s="1">
         <v>4.2019572E-7</v>
       </c>
       <c r="I24" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J24" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K24" s="1">
+        <v>4.2019572E-7</v>
+      </c>
+      <c r="L24" s="1">
         <v>1.2137457E+19</v>
       </c>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M24" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2099998E+19</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B25" s="1">
         <v>8.6058715000000004E-7</v>
       </c>
@@ -4415,25 +4770,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D25" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E25" s="1">
         <v>8.6058715000000004E-7</v>
       </c>
-      <c r="E25" s="1">
+      <c r="F25" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F25" s="1">
-        <v>8.6058715000000004E-7</v>
-      </c>
       <c r="G25" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H25" s="1">
         <v>8.6058715000000004E-7</v>
       </c>
       <c r="I25" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J25" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K25" s="1">
+        <v>8.6058715000000004E-7</v>
+      </c>
+      <c r="L25" s="1">
         <v>1.2137454E+19</v>
       </c>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M25" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2099995E+19</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B26" s="1">
         <v>9.9999999999999995E-7</v>
       </c>
@@ -4441,25 +4812,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D26" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E26" s="1">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="E26" s="1">
+      <c r="F26" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F26" s="1">
-        <v>9.9999999999999995E-7</v>
-      </c>
       <c r="G26" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H26" s="1">
         <v>9.9999999999999995E-7</v>
       </c>
       <c r="I26" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J26" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K26" s="1">
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="L26" s="1">
         <v>1.2137454E+19</v>
       </c>
-    </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M26" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2099995E+19</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B27" s="1">
         <v>1.8807829000000001E-6</v>
       </c>
@@ -4467,25 +4854,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D27" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E27" s="1">
         <v>1.8807829000000001E-6</v>
       </c>
-      <c r="E27" s="1">
+      <c r="F27" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F27" s="1">
-        <v>1.8807829000000001E-6</v>
-      </c>
       <c r="G27" s="1">
-        <v>1.1953784E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H27" s="1">
         <v>1.8807829000000001E-6</v>
       </c>
       <c r="I27" s="1">
+        <v>1.1953784E+19</v>
+      </c>
+      <c r="J27" s="1">
+        <f t="shared" si="2"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="K27" s="1">
+        <v>1.8807829000000001E-6</v>
+      </c>
+      <c r="L27" s="1">
         <v>1.2137449E+19</v>
       </c>
-    </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M27" s="1">
+        <f t="shared" si="3"/>
+        <v>1.209999E+19</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B28" s="1">
         <v>3.6423486E-6</v>
       </c>
@@ -4493,25 +4896,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D28" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E28" s="1">
         <v>3.6423486E-6</v>
       </c>
-      <c r="E28" s="1">
+      <c r="F28" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F28" s="1">
-        <v>3.6423486E-6</v>
-      </c>
       <c r="G28" s="1">
-        <v>1.1953783E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H28" s="1">
         <v>3.6423486E-6</v>
       </c>
       <c r="I28" s="1">
+        <v>1.1953783E+19</v>
+      </c>
+      <c r="J28" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099999E+19</v>
+      </c>
+      <c r="K28" s="1">
+        <v>3.6423486E-6</v>
+      </c>
+      <c r="L28" s="1">
         <v>1.213744E+19</v>
       </c>
-    </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M28" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2099981E+19</v>
+      </c>
+    </row>
+    <row r="29" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B29" s="1">
         <v>7.1654800999999996E-6</v>
       </c>
@@ -4519,25 +4938,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D29" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E29" s="1">
         <v>7.1654800999999996E-6</v>
       </c>
-      <c r="E29" s="1">
+      <c r="F29" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F29" s="1">
-        <v>7.1654800999999996E-6</v>
-      </c>
       <c r="G29" s="1">
-        <v>1.1953783E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H29" s="1">
         <v>7.1654800999999996E-6</v>
       </c>
       <c r="I29" s="1">
+        <v>1.1953783E+19</v>
+      </c>
+      <c r="J29" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099999E+19</v>
+      </c>
+      <c r="K29" s="1">
+        <v>7.1654800999999996E-6</v>
+      </c>
+      <c r="L29" s="1">
         <v>1.2137422E+19</v>
       </c>
-    </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M29" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2099963E+19</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B30" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -4545,25 +4980,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D30" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E30" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
-      <c r="E30" s="1">
+      <c r="F30" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F30" s="1">
-        <v>1.0000000000000001E-5</v>
-      </c>
       <c r="G30" s="1">
-        <v>1.1953783E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H30" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="I30" s="1">
+        <v>1.1953783E+19</v>
+      </c>
+      <c r="J30" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099999E+19</v>
+      </c>
+      <c r="K30" s="1">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="L30" s="1">
         <v>1.2137407E+19</v>
       </c>
-    </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M30" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2099948E+19</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B31" s="1">
         <v>1.7046262999999999E-5</v>
       </c>
@@ -4571,25 +5022,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D31" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E31" s="1">
         <v>1.7046262999999999E-5</v>
       </c>
-      <c r="E31" s="1">
+      <c r="F31" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F31" s="1">
-        <v>1.7046262999999999E-5</v>
-      </c>
       <c r="G31" s="1">
-        <v>1.1953783E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H31" s="1">
         <v>1.7046262999999999E-5</v>
       </c>
       <c r="I31" s="1">
+        <v>1.1953783E+19</v>
+      </c>
+      <c r="J31" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099999E+19</v>
+      </c>
+      <c r="K31" s="1">
+        <v>1.7046262999999999E-5</v>
+      </c>
+      <c r="L31" s="1">
         <v>1.213737E+19</v>
       </c>
-    </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M31" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2099911E+19</v>
+      </c>
+    </row>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B32" s="1">
         <v>3.1138788999999997E-5</v>
       </c>
@@ -4597,25 +5064,41 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D32" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E32" s="1">
         <v>3.1138788999999997E-5</v>
       </c>
-      <c r="E32" s="1">
+      <c r="F32" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F32" s="1">
-        <v>3.1138788999999997E-5</v>
-      </c>
       <c r="G32" s="1">
-        <v>1.1953782E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H32" s="1">
         <v>3.1138788999999997E-5</v>
       </c>
       <c r="I32" s="1">
+        <v>1.1953782E+19</v>
+      </c>
+      <c r="J32" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099998E+19</v>
+      </c>
+      <c r="K32" s="1">
+        <v>3.1138788999999997E-5</v>
+      </c>
+      <c r="L32" s="1">
         <v>1.2137298E+19</v>
       </c>
-    </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M32" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2099839E+19</v>
+      </c>
+    </row>
+    <row r="33" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B33" s="1">
         <v>5.9323841000000002E-5</v>
       </c>
@@ -4623,1036 +5106,1655 @@
         <v>1.1050604E+19</v>
       </c>
       <c r="D33" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E33" s="1">
         <v>5.9323841000000002E-5</v>
       </c>
-      <c r="E33" s="1">
+      <c r="F33" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F33" s="1">
-        <v>5.9323841000000002E-5</v>
-      </c>
       <c r="G33" s="1">
-        <v>1.195378E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H33" s="1">
         <v>5.9323841000000002E-5</v>
       </c>
       <c r="I33" s="1">
+        <v>1.195378E+19</v>
+      </c>
+      <c r="J33" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099996E+19</v>
+      </c>
+      <c r="K33" s="1">
+        <v>5.9323841000000002E-5</v>
+      </c>
+      <c r="L33" s="1">
         <v>1.2137155E+19</v>
       </c>
-    </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M33" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2099696E+19</v>
+      </c>
+    </row>
+    <row r="34" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B34">
         <v>1E-4</v>
       </c>
       <c r="C34" s="1">
         <v>1.1050604E+19</v>
       </c>
-      <c r="D34">
+      <c r="D34" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E34">
         <v>1E-4</v>
       </c>
-      <c r="E34" s="1">
+      <c r="F34" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F34">
-        <v>1E-4</v>
-      </c>
       <c r="G34" s="1">
-        <v>1.1953777E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H34">
         <v>1E-4</v>
       </c>
       <c r="I34" s="1">
+        <v>1.1953777E+19</v>
+      </c>
+      <c r="J34" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099993E+19</v>
+      </c>
+      <c r="K34">
+        <v>1E-4</v>
+      </c>
+      <c r="L34" s="1">
         <v>1.2136952E+19</v>
       </c>
-    </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M34" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2099493E+19</v>
+      </c>
+    </row>
+    <row r="35" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B35">
         <v>2.1274021E-4</v>
       </c>
       <c r="C35" s="1">
         <v>1.1050604E+19</v>
       </c>
-      <c r="D35">
+      <c r="D35" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E35">
         <v>2.1274021E-4</v>
       </c>
-      <c r="E35" s="1">
+      <c r="F35" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F35">
-        <v>2.1274021E-4</v>
-      </c>
       <c r="G35" s="1">
-        <v>1.195377E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H35">
         <v>2.1274021E-4</v>
       </c>
       <c r="I35" s="1">
+        <v>1.195377E+19</v>
+      </c>
+      <c r="J35" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099986E+19</v>
+      </c>
+      <c r="K35">
+        <v>2.1274021E-4</v>
+      </c>
+      <c r="L35" s="1">
         <v>1.2136416E+19</v>
       </c>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M35" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2098957E+19</v>
+      </c>
+    </row>
+    <row r="36" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B36">
         <v>4.3822061999999998E-4</v>
       </c>
       <c r="C36" s="1">
         <v>1.1050604E+19</v>
       </c>
-      <c r="D36">
+      <c r="D36" s="1">
+        <f t="shared" si="0"/>
+        <v>1.21E+19</v>
+      </c>
+      <c r="E36">
         <v>4.3822061999999998E-4</v>
       </c>
-      <c r="E36" s="1">
+      <c r="F36" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F36">
-        <v>4.3822061999999998E-4</v>
-      </c>
       <c r="G36" s="1">
-        <v>1.1953756E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H36">
         <v>4.3822061999999998E-4</v>
       </c>
       <c r="I36" s="1">
+        <v>1.1953756E+19</v>
+      </c>
+      <c r="J36" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099972E+19</v>
+      </c>
+      <c r="K36">
+        <v>4.3822061999999998E-4</v>
+      </c>
+      <c r="L36" s="1">
         <v>1.2135427E+19</v>
       </c>
-    </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M36" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2097968E+19</v>
+      </c>
+    </row>
+    <row r="37" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B37">
         <v>8.8918145E-4</v>
       </c>
       <c r="C37" s="1">
         <v>1.1050603E+19</v>
       </c>
-      <c r="D37">
+      <c r="D37" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2099999E+19</v>
+      </c>
+      <c r="E37">
         <v>8.8918145E-4</v>
       </c>
-      <c r="E37" s="1">
+      <c r="F37" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F37">
-        <v>8.8918145E-4</v>
-      </c>
       <c r="G37" s="1">
-        <v>1.1953729E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H37">
         <v>8.8918145E-4</v>
       </c>
       <c r="I37" s="1">
+        <v>1.1953729E+19</v>
+      </c>
+      <c r="J37" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099945E+19</v>
+      </c>
+      <c r="K37">
+        <v>8.8918145E-4</v>
+      </c>
+      <c r="L37" s="1">
         <v>1.2133695E+19</v>
       </c>
-    </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M37" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2096236E+19</v>
+      </c>
+    </row>
+    <row r="38" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B38">
         <v>1E-3</v>
       </c>
       <c r="C38" s="1">
         <v>1.1050603E+19</v>
       </c>
-      <c r="D38">
+      <c r="D38" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2099999E+19</v>
+      </c>
+      <c r="E38">
         <v>1E-3</v>
       </c>
-      <c r="E38" s="1">
+      <c r="F38" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F38">
-        <v>1E-3</v>
-      </c>
       <c r="G38" s="1">
-        <v>1.1953722E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H38">
         <v>1E-3</v>
       </c>
       <c r="I38" s="1">
+        <v>1.1953722E+19</v>
+      </c>
+      <c r="J38" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099938E+19</v>
+      </c>
+      <c r="K38">
+        <v>1E-3</v>
+      </c>
+      <c r="L38" s="1">
         <v>1.2133283E+19</v>
       </c>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M38" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2095824E+19</v>
+      </c>
+    </row>
+    <row r="39" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B39">
         <v>1.9019217E-3</v>
       </c>
       <c r="C39" s="1">
         <v>1.1050603E+19</v>
       </c>
-      <c r="D39">
+      <c r="D39" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2099999E+19</v>
+      </c>
+      <c r="E39">
         <v>1.9019217E-3</v>
       </c>
-      <c r="E39" s="1">
+      <c r="F39" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F39">
-        <v>1.9019217E-3</v>
-      </c>
       <c r="G39" s="1">
-        <v>1.1953666E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H39">
         <v>1.9019217E-3</v>
       </c>
       <c r="I39" s="1">
+        <v>1.1953666E+19</v>
+      </c>
+      <c r="J39" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099882E+19</v>
+      </c>
+      <c r="K39">
+        <v>1.9019217E-3</v>
+      </c>
+      <c r="L39" s="1">
         <v>1.2130518E+19</v>
       </c>
-    </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M39" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2093059E+19</v>
+      </c>
+    </row>
+    <row r="40" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B40">
         <v>3.7057650000000002E-3</v>
       </c>
       <c r="C40" s="1">
         <v>1.1050601E+19</v>
       </c>
-      <c r="D40">
+      <c r="D40" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2099997E+19</v>
+      </c>
+      <c r="E40">
         <v>3.7057650000000002E-3</v>
       </c>
-      <c r="E40" s="1">
+      <c r="F40" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F40">
-        <v>3.7057650000000002E-3</v>
-      </c>
       <c r="G40" s="1">
-        <v>1.1953558E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H40">
         <v>3.7057650000000002E-3</v>
       </c>
       <c r="I40" s="1">
+        <v>1.1953558E+19</v>
+      </c>
+      <c r="J40" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099774E+19</v>
+      </c>
+      <c r="K40">
+        <v>3.7057650000000002E-3</v>
+      </c>
+      <c r="L40" s="1">
         <v>1.2126289E+19</v>
       </c>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M40" s="1">
+        <f t="shared" si="3"/>
+        <v>1.208883E+19</v>
+      </c>
+    </row>
+    <row r="41" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B41">
         <v>7.3134515999999997E-3</v>
       </c>
       <c r="C41" s="1">
         <v>1.1050599E+19</v>
       </c>
-      <c r="D41">
+      <c r="D41" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2099995E+19</v>
+      </c>
+      <c r="E41">
         <v>7.3134515999999997E-3</v>
       </c>
-      <c r="E41" s="1">
+      <c r="F41" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F41">
-        <v>7.3134515999999997E-3</v>
-      </c>
       <c r="G41" s="1">
-        <v>1.1953346E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H41">
         <v>7.3134515999999997E-3</v>
       </c>
       <c r="I41" s="1">
+        <v>1.1953346E+19</v>
+      </c>
+      <c r="J41" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099562E+19</v>
+      </c>
+      <c r="K41">
+        <v>7.3134515999999997E-3</v>
+      </c>
+      <c r="L41" s="1">
         <v>1.2120324E+19</v>
       </c>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M41" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2082865E+19</v>
+      </c>
+    </row>
+    <row r="42" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B42">
         <v>0.01</v>
       </c>
       <c r="C42" s="1">
         <v>1.1050596E+19</v>
       </c>
-      <c r="D42">
+      <c r="D42" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2099992E+19</v>
+      </c>
+      <c r="E42">
         <v>0.01</v>
       </c>
-      <c r="E42" s="1">
+      <c r="F42" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F42">
-        <v>0.01</v>
-      </c>
       <c r="G42" s="1">
-        <v>1.1953191E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H42">
         <v>0.01</v>
       </c>
       <c r="I42" s="1">
+        <v>1.1953191E+19</v>
+      </c>
+      <c r="J42" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099407E+19</v>
+      </c>
+      <c r="K42">
+        <v>0.01</v>
+      </c>
+      <c r="L42" s="1">
         <v>1.2116741E+19</v>
       </c>
-    </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M42" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2079282E+19</v>
+      </c>
+    </row>
+    <row r="43" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B43">
         <v>1.7215372999999999E-2</v>
       </c>
       <c r="C43" s="1">
         <v>1.1050591E+19</v>
       </c>
-      <c r="D43">
+      <c r="D43" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2099987E+19</v>
+      </c>
+      <c r="E43">
         <v>1.7215372999999999E-2</v>
       </c>
-      <c r="E43" s="1">
+      <c r="F43" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F43">
-        <v>1.7215372999999999E-2</v>
-      </c>
       <c r="G43" s="1">
-        <v>1.1952797E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H43">
         <v>1.7215372999999999E-2</v>
       </c>
       <c r="I43" s="1">
+        <v>1.1952797E+19</v>
+      </c>
+      <c r="J43" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2099013E+19</v>
+      </c>
+      <c r="K43">
+        <v>1.7215372999999999E-2</v>
+      </c>
+      <c r="L43" s="1">
         <v>1.2110071E+19</v>
       </c>
-    </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M43" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2072612E+19</v>
+      </c>
+    </row>
+    <row r="44" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B44">
         <v>3.164612E-2</v>
       </c>
       <c r="C44" s="1">
         <v>1.105058E+19</v>
       </c>
-      <c r="D44">
+      <c r="D44" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2099976E+19</v>
+      </c>
+      <c r="E44">
         <v>3.164612E-2</v>
       </c>
-      <c r="E44" s="1">
+      <c r="F44" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F44">
-        <v>3.164612E-2</v>
-      </c>
       <c r="G44" s="1">
-        <v>1.1952073E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H44">
         <v>3.164612E-2</v>
       </c>
       <c r="I44" s="1">
+        <v>1.1952073E+19</v>
+      </c>
+      <c r="J44" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2098289E+19</v>
+      </c>
+      <c r="K44">
+        <v>3.164612E-2</v>
+      </c>
+      <c r="L44" s="1">
         <v>1.2101588E+19</v>
       </c>
-    </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M44" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2064129E+19</v>
+      </c>
+    </row>
+    <row r="45" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B45">
         <v>6.0507613000000002E-2</v>
       </c>
       <c r="C45" s="1">
         <v>1.1050558E+19</v>
       </c>
-      <c r="D45">
+      <c r="D45" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2099954E+19</v>
+      </c>
+      <c r="E45">
         <v>6.0507613000000002E-2</v>
       </c>
-      <c r="E45" s="1">
+      <c r="F45" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F45">
-        <v>6.0507613000000002E-2</v>
-      </c>
       <c r="G45" s="1">
-        <v>1.195081E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H45">
         <v>6.0507613000000002E-2</v>
       </c>
       <c r="I45" s="1">
+        <v>1.195081E+19</v>
+      </c>
+      <c r="J45" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2097026E+19</v>
+      </c>
+      <c r="K45">
+        <v>6.0507613000000002E-2</v>
+      </c>
+      <c r="L45" s="1">
         <v>1.20916E+19</v>
       </c>
-    </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M45" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2054141E+19</v>
+      </c>
+    </row>
+    <row r="46" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B46">
         <v>0.1</v>
       </c>
       <c r="C46" s="1">
         <v>1.1050528E+19</v>
       </c>
-      <c r="D46">
+      <c r="D46" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2099924E+19</v>
+      </c>
+      <c r="E46">
         <v>0.1</v>
       </c>
-      <c r="E46" s="1">
+      <c r="F46" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F46">
-        <v>0.1</v>
-      </c>
       <c r="G46" s="1">
-        <v>1.194932E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H46">
         <v>0.1</v>
       </c>
       <c r="I46" s="1">
+        <v>1.194932E+19</v>
+      </c>
+      <c r="J46" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2095536E+19</v>
+      </c>
+      <c r="K46">
+        <v>0.1</v>
+      </c>
+      <c r="L46" s="1">
         <v>1.208306E+19</v>
       </c>
-    </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M46" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2045601E+19</v>
+      </c>
+    </row>
+    <row r="47" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B47">
         <v>0.2</v>
       </c>
       <c r="C47" s="1">
         <v>1.1050453E+19</v>
       </c>
-      <c r="D47">
+      <c r="D47" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2099849E+19</v>
+      </c>
+      <c r="E47">
         <v>0.2</v>
       </c>
-      <c r="E47" s="1">
+      <c r="F47" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F47">
-        <v>0.2</v>
-      </c>
       <c r="G47" s="1">
-        <v>1.1946388E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H47">
         <v>0.2</v>
       </c>
       <c r="I47" s="1">
+        <v>1.1946388E+19</v>
+      </c>
+      <c r="J47" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2092604E+19</v>
+      </c>
+      <c r="K47">
+        <v>0.2</v>
+      </c>
+      <c r="L47" s="1">
         <v>1.2071348E+19</v>
       </c>
-    </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M47" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2033889E+19</v>
+      </c>
+    </row>
+    <row r="48" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B48">
         <v>0.43089195000000002</v>
       </c>
       <c r="C48" s="1">
         <v>1.1050287E+19</v>
       </c>
-      <c r="D48">
+      <c r="D48" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2099683E+19</v>
+      </c>
+      <c r="E48">
         <v>0.43089195000000002</v>
       </c>
-      <c r="E48" s="1">
+      <c r="F48" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F48">
-        <v>0.43089195000000002</v>
-      </c>
       <c r="G48" s="1">
-        <v>1.1941634E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H48">
         <v>0.43089195000000002</v>
       </c>
       <c r="I48" s="1">
+        <v>1.1941634E+19</v>
+      </c>
+      <c r="J48" s="1">
+        <f t="shared" si="2"/>
+        <v>1.208785E+19</v>
+      </c>
+      <c r="K48">
+        <v>0.43089195000000002</v>
+      </c>
+      <c r="L48" s="1">
         <v>1.2057637E+19</v>
       </c>
-    </row>
-    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M48" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2020178E+19</v>
+      </c>
+    </row>
+    <row r="49" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B49">
         <v>0.5</v>
       </c>
       <c r="C49" s="1">
         <v>1.1050238E+19</v>
       </c>
-      <c r="D49">
+      <c r="D49" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2099634E+19</v>
+      </c>
+      <c r="E49">
         <v>0.5</v>
       </c>
-      <c r="E49" s="1">
+      <c r="F49" s="1">
         <v>9.1386937E+18</v>
       </c>
-      <c r="F49">
-        <v>0.5</v>
-      </c>
       <c r="G49" s="1">
-        <v>1.1940351E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.21E+19</v>
       </c>
       <c r="H49">
         <v>0.5</v>
       </c>
       <c r="I49" s="1">
+        <v>1.1940351E+19</v>
+      </c>
+      <c r="J49" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2086567E+19</v>
+      </c>
+      <c r="K49">
+        <v>0.5</v>
+      </c>
+      <c r="L49" s="1">
         <v>1.2054261E+19</v>
       </c>
-    </row>
-    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M49" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2016802E+19</v>
+      </c>
+    </row>
+    <row r="50" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B50">
         <v>0.96178388999999997</v>
       </c>
       <c r="C50" s="1">
         <v>1.104993E+19</v>
       </c>
-      <c r="D50">
+      <c r="D50" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2099326E+19</v>
+      </c>
+      <c r="E50">
         <v>0.96178388999999997</v>
       </c>
-      <c r="E50" s="1">
+      <c r="F50" s="1">
         <v>9.1386936E+18</v>
       </c>
-      <c r="F50">
-        <v>0.96178388999999997</v>
-      </c>
       <c r="G50" s="1">
-        <v>1.1934505E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.20999999E+19</v>
       </c>
       <c r="H50">
         <v>0.96178388999999997</v>
       </c>
       <c r="I50" s="1">
+        <v>1.1934505E+19</v>
+      </c>
+      <c r="J50" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2080721E+19</v>
+      </c>
+      <c r="K50">
+        <v>0.96178388999999997</v>
+      </c>
+      <c r="L50" s="1">
         <v>1.2041111E+19</v>
       </c>
-    </row>
-    <row r="51" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M50" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2003652E+19</v>
+      </c>
+    </row>
+    <row r="51" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B51">
         <v>1</v>
       </c>
       <c r="C51" s="1">
         <v>1.1049904E+19</v>
       </c>
-      <c r="D51">
+      <c r="D51" s="1">
+        <f t="shared" si="0"/>
+        <v>1.20993E+19</v>
+      </c>
+      <c r="E51">
         <v>1</v>
       </c>
-      <c r="E51" s="1">
+      <c r="F51" s="1">
         <v>9.1386936E+18</v>
       </c>
-      <c r="F51">
-        <v>1</v>
-      </c>
       <c r="G51" s="1">
-        <v>1.1934038E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.20999999E+19</v>
       </c>
       <c r="H51">
         <v>1</v>
       </c>
       <c r="I51" s="1">
+        <v>1.1934038E+19</v>
+      </c>
+      <c r="J51" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2080254E+19</v>
+      </c>
+      <c r="K51">
+        <v>1</v>
+      </c>
+      <c r="L51" s="1">
         <v>1.2040077E+19</v>
       </c>
-    </row>
-    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M51" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2002618E+19</v>
+      </c>
+    </row>
+    <row r="52" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B52">
         <v>1.9235678</v>
       </c>
       <c r="C52" s="1">
         <v>1.1049351E+19</v>
       </c>
-      <c r="D52">
+      <c r="D52" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2098747E+19</v>
+      </c>
+      <c r="E52">
         <v>1.4617838999999999</v>
       </c>
-      <c r="E52" s="1">
+      <c r="F52" s="1">
         <v>9.1386936E+18</v>
       </c>
-      <c r="F52">
-        <v>1.9235678</v>
-      </c>
       <c r="G52" s="1">
-        <v>1.1926787E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.20999999E+19</v>
       </c>
       <c r="H52">
         <v>1.9235678</v>
       </c>
       <c r="I52" s="1">
+        <v>1.1926787E+19</v>
+      </c>
+      <c r="J52" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2073003E+19</v>
+      </c>
+      <c r="K52">
+        <v>1.9235678</v>
+      </c>
+      <c r="L52" s="1">
         <v>1.2024379E+19</v>
       </c>
-    </row>
-    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M52" s="1">
+        <f t="shared" si="3"/>
+        <v>1.198692E+19</v>
+      </c>
+    </row>
+    <row r="53" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B53">
         <v>2</v>
       </c>
       <c r="C53" s="1">
         <v>1.1049306E+19</v>
       </c>
-      <c r="D53">
+      <c r="D53" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2098702E+19</v>
+      </c>
+      <c r="E53">
         <v>2</v>
       </c>
-      <c r="E53" s="1">
+      <c r="F53" s="1">
         <v>9.1386935E+18</v>
       </c>
-      <c r="F53">
-        <v>2</v>
-      </c>
       <c r="G53" s="1">
-        <v>1.1926211E+19</v>
+        <f t="shared" si="1"/>
+        <v>1.20999998E+19</v>
       </c>
       <c r="H53">
         <v>2</v>
       </c>
       <c r="I53" s="1">
+        <v>1.1926211E+19</v>
+      </c>
+      <c r="J53" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2072427E+19</v>
+      </c>
+      <c r="K53">
+        <v>2</v>
+      </c>
+      <c r="L53" s="1">
         <v>1.2023133E+19</v>
       </c>
-    </row>
-    <row r="54" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M53" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1985674E+19</v>
+      </c>
+    </row>
+    <row r="54" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B54">
         <v>2.4617838999999999</v>
       </c>
       <c r="C54" s="1">
         <v>1.1049044E+19</v>
       </c>
-      <c r="D54">
+      <c r="D54" s="1">
+        <f t="shared" si="0"/>
+        <v>1.209844E+19</v>
+      </c>
+      <c r="E54">
         <v>2.8509943999999998</v>
       </c>
-      <c r="E54" s="1">
+      <c r="F54" s="1">
         <v>9.1386934E+18</v>
       </c>
-      <c r="F54">
+      <c r="G54" s="1">
+        <f t="shared" si="1"/>
+        <v>1.20999997E+19</v>
+      </c>
+      <c r="H54">
         <v>2.4617838999999999</v>
       </c>
-      <c r="G54" s="1">
+      <c r="I54" s="1">
         <v>1.1923333E+19</v>
       </c>
-      <c r="H54">
+      <c r="J54" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2069549E+19</v>
+      </c>
+      <c r="K54">
         <v>3.8471356000000001</v>
       </c>
-      <c r="I54" s="1">
+      <c r="L54" s="1">
         <v>1.2002551E+19</v>
       </c>
-    </row>
-    <row r="55" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M54" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1965092E+19</v>
+      </c>
+    </row>
+    <row r="55" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B55">
         <v>2.9235677999999998</v>
       </c>
       <c r="C55" s="1">
         <v>1.1048794E+19</v>
       </c>
-      <c r="D55">
+      <c r="D55" s="1">
+        <f t="shared" si="0"/>
+        <v>1.209819E+19</v>
+      </c>
+      <c r="E55">
         <v>3.4254972000000001</v>
       </c>
-      <c r="E55" s="1">
+      <c r="F55" s="1">
         <v>9.1386933E+18</v>
       </c>
-      <c r="F55">
+      <c r="G55" s="1">
+        <f t="shared" si="1"/>
+        <v>1.20999996E+19</v>
+      </c>
+      <c r="H55">
         <v>3.3853517000000002</v>
       </c>
-      <c r="G55" s="1">
+      <c r="I55" s="1">
         <v>1.191894E+19</v>
       </c>
-      <c r="H55">
+      <c r="J55" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2065156E+19</v>
+      </c>
+      <c r="K55">
         <v>4</v>
       </c>
-      <c r="I55" s="1">
+      <c r="L55" s="1">
         <v>1.2000904E+19</v>
       </c>
-    </row>
-    <row r="56" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M55" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1963445E+19</v>
+      </c>
+    </row>
+    <row r="56" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B56">
         <v>3.8471356000000001</v>
       </c>
       <c r="C56" s="1">
         <v>1.104833E+19</v>
       </c>
-      <c r="D56">
+      <c r="D56" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2097726E+19</v>
+      </c>
+      <c r="E56">
         <v>4</v>
       </c>
-      <c r="E56" s="1">
+      <c r="F56" s="1">
         <v>9.1386932E+18</v>
       </c>
-      <c r="F56">
+      <c r="G56" s="1">
+        <f t="shared" si="1"/>
+        <v>1.20999995E+19</v>
+      </c>
+      <c r="H56">
         <v>4</v>
       </c>
-      <c r="G56" s="1">
+      <c r="I56" s="1">
         <v>1.1916446E+19</v>
       </c>
-      <c r="H56">
+      <c r="J56" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2062662E+19</v>
+      </c>
+      <c r="K56">
         <v>4.9235677999999998</v>
       </c>
-      <c r="I56" s="1">
+      <c r="L56" s="1">
         <v>1.1992176E+19</v>
       </c>
-    </row>
-    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M56" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1954717E+19</v>
+      </c>
+    </row>
+    <row r="57" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B57">
         <v>4</v>
       </c>
       <c r="C57" s="1">
         <v>1.1048254E+19</v>
       </c>
-      <c r="D57">
+      <c r="D57" s="1">
+        <f t="shared" si="0"/>
+        <v>1.209765E+19</v>
+      </c>
+      <c r="E57">
         <v>5.8167374000000001</v>
       </c>
-      <c r="E57" s="1">
+      <c r="F57" s="1">
         <v>9.138693E+18</v>
       </c>
-      <c r="F57">
+      <c r="G57" s="1">
+        <f t="shared" si="1"/>
+        <v>1.20999993E+19</v>
+      </c>
+      <c r="H57">
         <v>4.9235677999999998</v>
       </c>
-      <c r="G57" s="1">
+      <c r="I57" s="1">
         <v>1.1913349E+19</v>
       </c>
-      <c r="H57">
+      <c r="J57" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2059565E+19</v>
+      </c>
+      <c r="K57">
         <v>5.8471355999999997</v>
       </c>
-      <c r="I57" s="1">
+      <c r="L57" s="1">
         <v>1.1984281E+19</v>
       </c>
-    </row>
-    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M57" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1946822E+19</v>
+      </c>
+    </row>
+    <row r="58" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B58">
         <v>4.9235677999999998</v>
       </c>
       <c r="C58" s="1">
         <v>1.1047825E+19</v>
       </c>
-      <c r="D58">
+      <c r="D58" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2097221E+19</v>
+      </c>
+      <c r="E58">
         <v>6.9083686999999996</v>
       </c>
-      <c r="E58" s="1">
+      <c r="F58" s="1">
         <v>9.1386929E+18</v>
       </c>
-      <c r="F58">
+      <c r="G58" s="1">
+        <f t="shared" si="1"/>
+        <v>1.20999992E+19</v>
+      </c>
+      <c r="H58">
         <v>5.3853517000000002</v>
       </c>
-      <c r="G58" s="1">
+      <c r="I58" s="1">
         <v>1.1911935E+19</v>
       </c>
-      <c r="H58">
+      <c r="J58" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2058151E+19</v>
+      </c>
+      <c r="K58">
         <v>7.6942710999999999</v>
       </c>
-      <c r="I58" s="1">
+      <c r="L58" s="1">
         <v>1.1970581E+19</v>
       </c>
-    </row>
-    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M58" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1933122E+19</v>
+      </c>
+    </row>
+    <row r="59" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B59">
         <v>6.7707033000000001</v>
       </c>
       <c r="C59" s="1">
         <v>1.1047054E+19</v>
       </c>
-      <c r="D59">
+      <c r="D59" s="1">
+        <f t="shared" si="0"/>
+        <v>1.209645E+19</v>
+      </c>
+      <c r="E59">
         <v>8</v>
       </c>
-      <c r="E59" s="1">
+      <c r="F59" s="1">
         <v>9.1386927E+18</v>
       </c>
-      <c r="F59">
+      <c r="G59" s="1">
+        <f t="shared" si="1"/>
+        <v>1.2099999E+19</v>
+      </c>
+      <c r="H59">
         <v>6.3089195</v>
       </c>
-      <c r="G59" s="1">
+      <c r="I59" s="1">
         <v>1.1909499E+19</v>
       </c>
-      <c r="H59">
+      <c r="J59" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2055715E+19</v>
+      </c>
+      <c r="K59">
         <v>8</v>
       </c>
-      <c r="I59" s="1">
+      <c r="L59" s="1">
         <v>1.1968366E+19</v>
       </c>
-    </row>
-    <row r="60" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M59" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1930907E+19</v>
+      </c>
+    </row>
+    <row r="60" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B60">
         <v>8</v>
       </c>
       <c r="C60" s="1">
         <v>1.1046573E+19</v>
       </c>
-      <c r="D60">
+      <c r="D60" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2095969E+19</v>
+      </c>
+      <c r="E60">
         <v>9.0916312999999995</v>
       </c>
-      <c r="E60" s="1">
+      <c r="F60" s="1">
         <v>9.1386926E+18</v>
       </c>
-      <c r="F60">
+      <c r="G60" s="1">
+        <f t="shared" si="1"/>
+        <v>1.20999989E+19</v>
+      </c>
+      <c r="H60">
         <v>8</v>
       </c>
-      <c r="G60" s="1">
+      <c r="I60" s="1">
         <v>1.19059E+19</v>
       </c>
-      <c r="H60">
+      <c r="J60" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2052116E+19</v>
+      </c>
+      <c r="K60">
         <v>11.694271000000001</v>
       </c>
-      <c r="I60" s="1">
+      <c r="L60" s="1">
         <v>1.1946294E+19</v>
       </c>
-    </row>
-    <row r="61" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M60" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1908835E+19</v>
+      </c>
+    </row>
+    <row r="61" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B61">
         <v>9.8471355999999997</v>
       </c>
       <c r="C61" s="1">
         <v>1.1045909E+19</v>
       </c>
-      <c r="D61">
+      <c r="D61" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2095305E+19</v>
+      </c>
+      <c r="E61">
         <v>9.6374469999999999</v>
       </c>
-      <c r="E61" s="1">
+      <c r="F61" s="1">
         <v>9.1386925E+18</v>
       </c>
-      <c r="F61">
+      <c r="G61" s="1">
+        <f t="shared" si="1"/>
+        <v>1.20999988E+19</v>
+      </c>
+      <c r="H61">
         <v>11.694271000000001</v>
       </c>
-      <c r="G61" s="1">
+      <c r="I61" s="1">
         <v>1.1900226E+19</v>
       </c>
-      <c r="H61">
+      <c r="J61" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2046442E+19</v>
+      </c>
+      <c r="K61">
         <v>12.770702999999999</v>
       </c>
-      <c r="I61" s="1">
+      <c r="L61" s="1">
         <v>1.1940209E+19</v>
       </c>
-    </row>
-    <row r="62" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M61" s="1">
+        <f t="shared" si="3"/>
+        <v>1.190275E+19</v>
+      </c>
+    </row>
+    <row r="62" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B62">
         <v>10.770702999999999</v>
       </c>
       <c r="C62" s="1">
         <v>1.104559E+19</v>
       </c>
-      <c r="D62">
+      <c r="D62" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2094986E+19</v>
+      </c>
+      <c r="E62">
         <v>10.183263</v>
       </c>
-      <c r="E62" s="1">
+      <c r="F62" s="1">
         <v>9.1386925E+18</v>
       </c>
-      <c r="F62">
+      <c r="G62" s="1">
+        <f t="shared" si="1"/>
+        <v>1.20999988E+19</v>
+      </c>
+      <c r="H62">
         <v>12.770702999999999</v>
       </c>
-      <c r="G62" s="1">
+      <c r="I62" s="1">
         <v>1.1898724E+19</v>
       </c>
-      <c r="H62">
+      <c r="J62" s="1">
+        <f t="shared" si="2"/>
+        <v>1.204494E+19</v>
+      </c>
+      <c r="K62">
         <v>14.923568</v>
       </c>
-      <c r="I62" s="1">
+      <c r="L62" s="1">
         <v>1.1929154E+19</v>
       </c>
-    </row>
-    <row r="63" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M62" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1891695E+19</v>
+      </c>
+    </row>
+    <row r="63" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B63">
         <v>11.694271000000001</v>
       </c>
       <c r="C63" s="1">
         <v>1.1045282E+19</v>
       </c>
-      <c r="D63">
+      <c r="D63" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2094678E+19</v>
+      </c>
+      <c r="E63">
         <v>10.729077999999999</v>
       </c>
-      <c r="E63" s="1">
+      <c r="F63" s="1">
         <v>9.1386924E+18</v>
       </c>
-      <c r="F63">
+      <c r="G63" s="1">
+        <f t="shared" si="1"/>
+        <v>1.20999987E+19</v>
+      </c>
+      <c r="H63">
         <v>13.308918999999999</v>
       </c>
-      <c r="G63" s="1">
+      <c r="I63" s="1">
         <v>1.1898008E+19</v>
       </c>
-      <c r="H63">
+      <c r="J63" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2044224E+19</v>
+      </c>
+      <c r="K63">
         <v>16</v>
       </c>
-      <c r="I63" s="1">
+      <c r="L63" s="1">
         <v>1.192388E+19</v>
       </c>
-    </row>
-    <row r="64" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M63" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1886421E+19</v>
+      </c>
+    </row>
+    <row r="64" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B64">
         <v>13.541407</v>
       </c>
       <c r="C64" s="1">
         <v>1.1044707E+19</v>
       </c>
-      <c r="D64">
+      <c r="D64" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2094103E+19</v>
+      </c>
+      <c r="E64">
         <v>11.274894</v>
       </c>
-      <c r="E64" s="1">
+      <c r="F64" s="1">
         <v>9.1386923E+18</v>
       </c>
-      <c r="F64">
+      <c r="G64" s="1">
+        <f t="shared" si="1"/>
+        <v>1.20999986E+19</v>
+      </c>
+      <c r="H64">
         <v>14.385351999999999</v>
       </c>
-      <c r="G64" s="1">
+      <c r="I64" s="1">
         <v>1.189669E+19</v>
       </c>
-      <c r="H64">
+      <c r="J64" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2042906E+19</v>
+      </c>
+      <c r="K64">
         <v>17.076432</v>
       </c>
-      <c r="I64" s="1">
+      <c r="L64" s="1">
         <v>1.1918836E+19</v>
       </c>
-    </row>
-    <row r="65" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M64" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1881377E+19</v>
+      </c>
+    </row>
+    <row r="65" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B65">
         <v>14.770702999999999</v>
       </c>
       <c r="C65" s="1">
         <v>1.104434E+19</v>
       </c>
-      <c r="D65">
+      <c r="D65" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2093736E+19</v>
+      </c>
+      <c r="E65">
         <v>11.82071</v>
       </c>
-      <c r="E65" s="1">
+      <c r="F65" s="1">
         <v>9.1386923E+18</v>
       </c>
-      <c r="F65">
+      <c r="G65" s="1">
+        <f t="shared" si="1"/>
+        <v>1.20999986E+19</v>
+      </c>
+      <c r="H65">
         <v>15.192676000000001</v>
       </c>
-      <c r="G65" s="1">
+      <c r="I65" s="1">
         <v>1.1895759E+19</v>
       </c>
-      <c r="H65">
+      <c r="J65" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2041975E+19</v>
+      </c>
+      <c r="K65">
         <v>19.229296999999999</v>
       </c>
-      <c r="I65" s="1">
+      <c r="L65" s="1">
         <v>1.1909537E+19</v>
       </c>
-    </row>
-    <row r="66" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M65" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1872078E+19</v>
+      </c>
+    </row>
+    <row r="66" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B66">
         <v>16</v>
       </c>
       <c r="C66" s="1">
         <v>1.1043987E+19</v>
       </c>
-      <c r="D66">
+      <c r="D66" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2093383E+19</v>
+      </c>
+      <c r="E66">
         <v>12.366524999999999</v>
       </c>
-      <c r="E66" s="1">
+      <c r="F66" s="1">
         <v>9.1386922E+18</v>
       </c>
-      <c r="F66">
+      <c r="G66" s="1">
+        <f t="shared" si="1"/>
+        <v>1.20999985E+19</v>
+      </c>
+      <c r="H66">
         <v>16</v>
       </c>
-      <c r="G66" s="1">
+      <c r="I66" s="1">
         <v>1.1894878E+19</v>
       </c>
-      <c r="H66">
+      <c r="J66" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2041094E+19</v>
+      </c>
+      <c r="K66">
         <v>21.382161</v>
       </c>
-      <c r="I66" s="1">
+      <c r="L66" s="1">
         <v>1.1900924E+19</v>
       </c>
-    </row>
-    <row r="67" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M66" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1863465E+19</v>
+      </c>
+    </row>
+    <row r="67" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B67" t="s">
         <v>14</v>
       </c>
       <c r="C67" t="s">
         <v>14</v>
       </c>
-      <c r="D67">
+      <c r="D67" s="1"/>
+      <c r="E67">
         <v>13.458157</v>
       </c>
-      <c r="E67" s="1">
+      <c r="F67" s="1">
         <v>9.1386921E+18</v>
       </c>
-      <c r="F67">
+      <c r="G67" s="1">
+        <f t="shared" si="1"/>
+        <v>1.20999984E+19</v>
+      </c>
+      <c r="H67">
         <v>18.552983000000001</v>
       </c>
-      <c r="G67" s="1">
+      <c r="I67" s="1">
         <v>1.1892472E+19</v>
       </c>
-      <c r="H67">
+      <c r="J67" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2038688E+19</v>
+      </c>
+      <c r="K67">
         <v>22.458593</v>
       </c>
-      <c r="I67" s="1">
+      <c r="L67" s="1">
         <v>1.1896778E+19</v>
       </c>
-    </row>
-    <row r="68" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M67" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1859319E+19</v>
+      </c>
+    </row>
+    <row r="68" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
         <v>14</v>
       </c>
       <c r="C68" t="s">
         <v>14</v>
       </c>
-      <c r="D68">
+      <c r="D68" s="1"/>
+      <c r="E68">
         <v>14.003971999999999</v>
       </c>
-      <c r="E68" s="1">
+      <c r="F68" s="1">
         <v>9.138692E+18</v>
       </c>
-      <c r="F68">
+      <c r="G68" s="1">
+        <f t="shared" ref="G68:G72" si="4">12100000000000000000-F$3+F68</f>
+        <v>1.20999983E+19</v>
+      </c>
+      <c r="H68">
         <v>19.191229</v>
       </c>
-      <c r="G68" s="1">
+      <c r="I68" s="1">
         <v>1.1891893E+19</v>
       </c>
-      <c r="H68">
+      <c r="J68" s="1">
+        <f t="shared" ref="J68:J72" si="5">12100000000000000000-I$3+I68</f>
+        <v>1.2038109E+19</v>
+      </c>
+      <c r="K68">
         <v>22.996808999999999</v>
       </c>
-      <c r="I68" s="1">
+      <c r="L68" s="1">
         <v>1.1894743E+19</v>
       </c>
-    </row>
-    <row r="69" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M68" s="1">
+        <f t="shared" ref="M68:M72" si="6">12100000000000000000-L$3+L68</f>
+        <v>1.1857284E+19</v>
+      </c>
+    </row>
+    <row r="69" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
         <v>14</v>
       </c>
       <c r="C69" t="s">
         <v>14</v>
       </c>
-      <c r="D69">
+      <c r="D69" s="1"/>
+      <c r="E69">
         <v>14.549787999999999</v>
       </c>
-      <c r="E69" s="1">
+      <c r="F69" s="1">
         <v>9.1386919E+18</v>
       </c>
-      <c r="F69">
+      <c r="G69" s="1">
+        <f t="shared" si="4"/>
+        <v>1.20999982E+19</v>
+      </c>
+      <c r="H69">
         <v>19.829474999999999</v>
       </c>
-      <c r="G69" s="1">
+      <c r="I69" s="1">
         <v>1.1891333E+19</v>
       </c>
-      <c r="H69">
+      <c r="J69" s="1">
+        <f t="shared" si="5"/>
+        <v>1.2037549E+19</v>
+      </c>
+      <c r="K69">
         <v>24.073242</v>
       </c>
-      <c r="I69" s="1">
+      <c r="L69" s="1">
         <v>1.1890818E+19</v>
       </c>
-    </row>
-    <row r="70" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M69" s="1">
+        <f t="shared" si="6"/>
+        <v>1.1853359E+19</v>
+      </c>
+    </row>
+    <row r="70" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
         <v>14</v>
       </c>
       <c r="C70" t="s">
         <v>14</v>
       </c>
-      <c r="D70">
+      <c r="D70" s="1"/>
+      <c r="E70">
         <v>15.095603000000001</v>
       </c>
-      <c r="E70" s="1">
+      <c r="F70" s="1">
         <v>9.1386919E+18</v>
       </c>
-      <c r="F70">
+      <c r="G70" s="1">
+        <f t="shared" si="4"/>
+        <v>1.20999982E+19</v>
+      </c>
+      <c r="H70">
         <v>21.105965999999999</v>
       </c>
-      <c r="G70" s="1">
+      <c r="I70" s="1">
         <v>1.1890285E+19</v>
       </c>
-      <c r="H70">
+      <c r="J70" s="1">
+        <f t="shared" si="5"/>
+        <v>1.2036501E+19</v>
+      </c>
+      <c r="K70">
         <v>25.149674000000001</v>
       </c>
-      <c r="I70" s="1">
+      <c r="L70" s="1">
         <v>1.188703E+19</v>
       </c>
-    </row>
-    <row r="71" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M70" s="1">
+        <f t="shared" si="6"/>
+        <v>1.1849571E+19</v>
+      </c>
+    </row>
+    <row r="71" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B71" t="s">
         <v>14</v>
       </c>
       <c r="C71" t="s">
         <v>14</v>
       </c>
-      <c r="D71">
+      <c r="D71" s="1"/>
+      <c r="E71">
         <v>16</v>
       </c>
-      <c r="E71" s="1">
+      <c r="F71" s="1">
         <v>9.1386918E+18</v>
       </c>
-      <c r="F71">
+      <c r="G71" s="1">
+        <f t="shared" si="4"/>
+        <v>1.20999981E+19</v>
+      </c>
+      <c r="H71">
         <v>22.382458</v>
       </c>
-      <c r="G71" s="1">
+      <c r="I71" s="1">
         <v>1.18893E+19</v>
       </c>
-      <c r="H71">
+      <c r="J71" s="1">
+        <f t="shared" si="5"/>
+        <v>1.2035516E+19</v>
+      </c>
+      <c r="K71">
         <v>26.226106000000001</v>
       </c>
-      <c r="I71" s="1">
+      <c r="L71" s="1">
         <v>1.188337E+19</v>
       </c>
-    </row>
-    <row r="72" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="M71" s="1">
+        <f t="shared" si="6"/>
+        <v>1.1845911E+19</v>
+      </c>
+    </row>
+    <row r="72" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B72" t="s">
         <v>14</v>
       </c>
       <c r="C72" t="s">
         <v>14</v>
       </c>
-      <c r="D72">
+      <c r="D72" s="1"/>
+      <c r="E72">
         <v>16.545815999999999</v>
       </c>
-      <c r="E72" s="1">
+      <c r="F72" s="1">
         <v>9.1386917E+18</v>
       </c>
-      <c r="F72" t="s">
+      <c r="G72" s="1">
+        <f t="shared" si="4"/>
+        <v>1.2099998E+19</v>
+      </c>
+      <c r="H72" t="s">
         <v>14</v>
       </c>
-      <c r="G72" t="s">
+      <c r="I72" t="s">
         <v>14</v>
       </c>
-      <c r="H72">
+      <c r="J72" s="1"/>
+      <c r="K72">
         <v>26.764322</v>
       </c>
-      <c r="I72" s="1">
+      <c r="L72" s="1">
         <v>1.1881571E+19</v>
+      </c>
+      <c r="M72" s="1">
+        <f t="shared" si="6"/>
+        <v>1.1844112E+19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>